<commit_message>
Membuat Nama Perusahaan dan Nama Proyek dinamis berdasarkan input Excel
</commit_message>
<xml_diff>
--- a/Template_Dashboard_v2.xlsx
+++ b/Template_Dashboard_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://365mic-my.sharepoint.com/personal/ipanjez_365mic_onmicrosoft_com/Documents/Learn/Coding/Dashboard Proyek Soda Ash/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="113" documentId="11_FBD64D39D349D756657D4B1399D967C19B799422" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{25C4878D-1B90-4CEB-854D-FFE7585F0910}"/>
+  <xr:revisionPtr revIDLastSave="125" documentId="11_FBD64D39D349D756657D4B1399D967C19B799422" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B5E05A04-893E-4398-BD0D-0B79E4C17403}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -511,7 +511,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="523" uniqueCount="408">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="527" uniqueCount="412">
   <si>
     <t>EXECUTIVE ACTION TRACKER — DIREKSI / PROJECT STEERING COMMITTEE (PSC)</t>
   </si>
@@ -1739,6 +1739,18 @@
   </si>
   <si>
     <t>C -&gt;</t>
+  </si>
+  <si>
+    <t>Nama Perusahaan</t>
+  </si>
+  <si>
+    <t>Perusahaan X</t>
+  </si>
+  <si>
+    <t>Nama Proyek</t>
+  </si>
+  <si>
+    <t>Proyek X</t>
   </si>
 </sst>
 </file>
@@ -1749,7 +1761,7 @@
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
     <numFmt numFmtId="165" formatCode="#,##0.0;\(#,##0.0\)"/>
   </numFmts>
-  <fonts count="52" x14ac:knownFonts="1">
+  <fonts count="54" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2092,8 +2104,22 @@
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF0070C0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="30">
+  <fills count="31">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2266,6 +2292,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFEAEAEA"/>
         <bgColor rgb="FFEAEAEA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -2467,7 +2499,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="198">
+  <cellXfs count="200">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -2763,207 +2795,207 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="51" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="28" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="8" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="1" fontId="18" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="24" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="18" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="17" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="15" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="18" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="23" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="24" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="24" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="24" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="18" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="18" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="24" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="8" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="17" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="10" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="24" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="23" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="24" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="24" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="15" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="37" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -2976,6 +3008,8 @@
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="52" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="53" fillId="30" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3382,7 +3416,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:23" ht="30" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B1" s="167" t="s">
+      <c r="B1" s="182" t="s">
         <v>378</v>
       </c>
       <c r="C1" s="116"/>
@@ -3408,9 +3442,9 @@
       <c r="W1" s="118"/>
     </row>
     <row r="2" spans="2:23" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B2" s="186" t="str">
+      <c r="B2" s="152" t="str">
         <f ca="1">"Reporting Period: "&amp;Input_Bulanan!D5&amp;"   |   Status: "&amp;Input_Bulanan!F5&amp;"   |   Dicetak: "&amp;TEXT(TODAY(),"DD-MM-YYYY")</f>
-        <v>Reporting Period: Agustus 2026   |   Status: DRAFT   |   Dicetak: 18-07-2026</v>
+        <v>Reporting Period: Agustus 2026   |   Status: DRAFT   |   Dicetak: 20-07-2026</v>
       </c>
       <c r="C2" s="114"/>
       <c r="D2" s="114"/>
@@ -3436,7 +3470,7 @@
     </row>
     <row r="3" spans="2:23" ht="6" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="4" spans="2:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B4" s="138" t="s">
+      <c r="B4" s="153" t="s">
         <v>47</v>
       </c>
       <c r="C4" s="116"/>
@@ -3449,7 +3483,7 @@
       <c r="J4" s="116"/>
       <c r="K4" s="116"/>
       <c r="L4" s="118"/>
-      <c r="M4" s="138" t="s">
+      <c r="M4" s="153" t="s">
         <v>48</v>
       </c>
       <c r="N4" s="116"/>
@@ -3464,14 +3498,14 @@
       <c r="W4" s="118"/>
     </row>
     <row r="5" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B5" s="152" t="s">
+      <c r="B5" s="162" t="s">
         <v>49</v>
       </c>
       <c r="C5" s="116"/>
       <c r="D5" s="116"/>
       <c r="E5" s="116"/>
       <c r="F5" s="118"/>
-      <c r="G5" s="152" t="s">
+      <c r="G5" s="162" t="s">
         <v>50</v>
       </c>
       <c r="H5" s="116"/>
@@ -3479,14 +3513,14 @@
       <c r="J5" s="116"/>
       <c r="K5" s="116"/>
       <c r="L5" s="118"/>
-      <c r="M5" s="152" t="s">
+      <c r="M5" s="162" t="s">
         <v>51</v>
       </c>
       <c r="N5" s="116"/>
       <c r="O5" s="116"/>
       <c r="P5" s="116"/>
       <c r="Q5" s="118"/>
-      <c r="R5" s="188" t="s">
+      <c r="R5" s="147" t="s">
         <v>52</v>
       </c>
       <c r="S5" s="116"/>
@@ -3496,33 +3530,33 @@
       <c r="W5" s="118"/>
     </row>
     <row r="6" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B6" s="154">
+      <c r="B6" s="192">
         <f>((IF(Input_Bulanan!D11&gt;=1,100,Input_Bulanan!D11*100)*0.2)+(IF(Input_Bulanan!D13&gt;=1,100,Input_Bulanan!D13*100)*0.2)+(Input_Bulanan!D22*100*0.2)+(Input_Bulanan!D29*100*0.2)+(Input_Bulanan!D38*100*0.2))/100</f>
         <v>0.69100000000000006</v>
       </c>
-      <c r="C6" s="142"/>
-      <c r="D6" s="142"/>
-      <c r="E6" s="142"/>
-      <c r="F6" s="143"/>
-      <c r="G6" s="173" t="s">
+      <c r="C6" s="156"/>
+      <c r="D6" s="156"/>
+      <c r="E6" s="156"/>
+      <c r="F6" s="142"/>
+      <c r="G6" s="160" t="s">
         <v>53</v>
       </c>
-      <c r="H6" s="142"/>
-      <c r="I6" s="142"/>
-      <c r="J6" s="142"/>
-      <c r="K6" s="148">
+      <c r="H6" s="156"/>
+      <c r="I6" s="156"/>
+      <c r="J6" s="156"/>
+      <c r="K6" s="141">
         <f>Input_Bulanan!D22</f>
         <v>6.7000000000000004E-2</v>
       </c>
-      <c r="L6" s="143"/>
-      <c r="M6" s="187" t="str">
+      <c r="L6" s="142"/>
+      <c r="M6" s="155" t="str">
         <f>Input_Bulanan!D45</f>
         <v>Moderate</v>
       </c>
-      <c r="N6" s="142"/>
-      <c r="O6" s="142"/>
-      <c r="P6" s="142"/>
-      <c r="Q6" s="143"/>
+      <c r="N6" s="156"/>
+      <c r="O6" s="156"/>
+      <c r="P6" s="156"/>
+      <c r="Q6" s="142"/>
       <c r="R6" s="1" t="s">
         <v>402</v>
       </c>
@@ -3548,22 +3582,22 @@
       </c>
     </row>
     <row r="7" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B7" s="155"/>
+      <c r="B7" s="157"/>
       <c r="C7" s="114"/>
       <c r="D7" s="114"/>
       <c r="E7" s="114"/>
-      <c r="F7" s="156"/>
-      <c r="G7" s="144"/>
-      <c r="H7" s="145"/>
-      <c r="I7" s="145"/>
-      <c r="J7" s="145"/>
-      <c r="K7" s="145"/>
-      <c r="L7" s="146"/>
-      <c r="M7" s="155"/>
+      <c r="F7" s="158"/>
+      <c r="G7" s="159"/>
+      <c r="H7" s="143"/>
+      <c r="I7" s="143"/>
+      <c r="J7" s="143"/>
+      <c r="K7" s="143"/>
+      <c r="L7" s="144"/>
+      <c r="M7" s="157"/>
       <c r="N7" s="114"/>
       <c r="O7" s="114"/>
       <c r="P7" s="114"/>
-      <c r="Q7" s="156"/>
+      <c r="Q7" s="158"/>
       <c r="R7" s="1" t="s">
         <v>403</v>
       </c>
@@ -3589,27 +3623,27 @@
       </c>
     </row>
     <row r="8" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B8" s="155"/>
+      <c r="B8" s="157"/>
       <c r="C8" s="114"/>
       <c r="D8" s="114"/>
       <c r="E8" s="114"/>
-      <c r="F8" s="156"/>
-      <c r="G8" s="173" t="s">
+      <c r="F8" s="158"/>
+      <c r="G8" s="160" t="s">
         <v>54</v>
       </c>
-      <c r="H8" s="142"/>
-      <c r="I8" s="142"/>
-      <c r="J8" s="142"/>
-      <c r="K8" s="148">
+      <c r="H8" s="156"/>
+      <c r="I8" s="156"/>
+      <c r="J8" s="156"/>
+      <c r="K8" s="141">
         <f>Input_Bulanan!D29</f>
         <v>0.76800000000000002</v>
       </c>
-      <c r="L8" s="143"/>
-      <c r="M8" s="155"/>
+      <c r="L8" s="142"/>
+      <c r="M8" s="157"/>
       <c r="N8" s="114"/>
       <c r="O8" s="114"/>
       <c r="P8" s="114"/>
-      <c r="Q8" s="156"/>
+      <c r="Q8" s="158"/>
       <c r="R8" s="1" t="s">
         <v>404</v>
       </c>
@@ -3635,22 +3669,22 @@
       </c>
     </row>
     <row r="9" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B9" s="144"/>
-      <c r="C9" s="145"/>
-      <c r="D9" s="145"/>
-      <c r="E9" s="145"/>
-      <c r="F9" s="146"/>
-      <c r="G9" s="144"/>
-      <c r="H9" s="145"/>
-      <c r="I9" s="145"/>
-      <c r="J9" s="145"/>
-      <c r="K9" s="145"/>
-      <c r="L9" s="146"/>
-      <c r="M9" s="144"/>
-      <c r="N9" s="145"/>
-      <c r="O9" s="145"/>
-      <c r="P9" s="145"/>
-      <c r="Q9" s="146"/>
+      <c r="B9" s="159"/>
+      <c r="C9" s="143"/>
+      <c r="D9" s="143"/>
+      <c r="E9" s="143"/>
+      <c r="F9" s="144"/>
+      <c r="G9" s="159"/>
+      <c r="H9" s="143"/>
+      <c r="I9" s="143"/>
+      <c r="J9" s="143"/>
+      <c r="K9" s="143"/>
+      <c r="L9" s="144"/>
+      <c r="M9" s="159"/>
+      <c r="N9" s="143"/>
+      <c r="O9" s="143"/>
+      <c r="P9" s="143"/>
+      <c r="Q9" s="144"/>
       <c r="R9" s="1" t="s">
         <v>405</v>
       </c>
@@ -3676,33 +3710,33 @@
       </c>
     </row>
     <row r="10" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B10" s="141" t="str">
+      <c r="B10" s="191" t="str">
         <f>IF(B6&gt;=0.9,"HIJAU - SEHAT",IF(B6&gt;=0.75,"KUNING - PANTAU",IF(B6&gt;=0.6,"ORANYE - WASPADA","MERAH - KRITIS")))</f>
         <v>ORANYE - WASPADA</v>
       </c>
-      <c r="C10" s="142"/>
-      <c r="D10" s="142"/>
-      <c r="E10" s="142"/>
-      <c r="F10" s="143"/>
-      <c r="G10" s="173" t="s">
+      <c r="C10" s="156"/>
+      <c r="D10" s="156"/>
+      <c r="E10" s="156"/>
+      <c r="F10" s="142"/>
+      <c r="G10" s="160" t="s">
         <v>55</v>
       </c>
-      <c r="H10" s="142"/>
-      <c r="I10" s="142"/>
-      <c r="J10" s="142"/>
-      <c r="K10" s="148">
+      <c r="H10" s="156"/>
+      <c r="I10" s="156"/>
+      <c r="J10" s="156"/>
+      <c r="K10" s="141">
         <f>Input_Bulanan!D38</f>
         <v>0.62</v>
       </c>
-      <c r="L10" s="143"/>
-      <c r="M10" s="175" t="str">
+      <c r="L10" s="142"/>
+      <c r="M10" s="168" t="str">
         <f>"Skor Komposit: "&amp;TEXT(Input_Bulanan!D44,"0,00")&amp;" / 100"</f>
         <v>Skor Komposit: 45,80 / 100</v>
       </c>
-      <c r="N10" s="142"/>
-      <c r="O10" s="142"/>
-      <c r="P10" s="142"/>
-      <c r="Q10" s="143"/>
+      <c r="N10" s="156"/>
+      <c r="O10" s="156"/>
+      <c r="P10" s="156"/>
+      <c r="Q10" s="142"/>
       <c r="R10" s="1" t="s">
         <v>406</v>
       </c>
@@ -3728,22 +3762,22 @@
       </c>
     </row>
     <row r="11" spans="2:23" ht="12" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B11" s="144"/>
-      <c r="C11" s="145"/>
-      <c r="D11" s="145"/>
-      <c r="E11" s="145"/>
-      <c r="F11" s="146"/>
-      <c r="G11" s="144"/>
-      <c r="H11" s="145"/>
-      <c r="I11" s="145"/>
-      <c r="J11" s="145"/>
-      <c r="K11" s="145"/>
-      <c r="L11" s="146"/>
-      <c r="M11" s="144"/>
-      <c r="N11" s="145"/>
-      <c r="O11" s="145"/>
-      <c r="P11" s="145"/>
-      <c r="Q11" s="146"/>
+      <c r="B11" s="159"/>
+      <c r="C11" s="143"/>
+      <c r="D11" s="143"/>
+      <c r="E11" s="143"/>
+      <c r="F11" s="144"/>
+      <c r="G11" s="159"/>
+      <c r="H11" s="143"/>
+      <c r="I11" s="143"/>
+      <c r="J11" s="143"/>
+      <c r="K11" s="143"/>
+      <c r="L11" s="144"/>
+      <c r="M11" s="159"/>
+      <c r="N11" s="143"/>
+      <c r="O11" s="143"/>
+      <c r="P11" s="143"/>
+      <c r="Q11" s="144"/>
       <c r="R11" s="7" t="s">
         <v>407</v>
       </c>
@@ -3764,14 +3798,14 @@
       </c>
     </row>
     <row r="12" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B12" s="152" t="s">
+      <c r="B12" s="162" t="s">
         <v>56</v>
       </c>
       <c r="C12" s="116"/>
       <c r="D12" s="116"/>
       <c r="E12" s="116"/>
       <c r="F12" s="118"/>
-      <c r="G12" s="152" t="s">
+      <c r="G12" s="162" t="s">
         <v>57</v>
       </c>
       <c r="H12" s="116"/>
@@ -3779,14 +3813,14 @@
       <c r="J12" s="116"/>
       <c r="K12" s="116"/>
       <c r="L12" s="118"/>
-      <c r="M12" s="152" t="s">
+      <c r="M12" s="162" t="s">
         <v>58</v>
       </c>
       <c r="N12" s="116"/>
       <c r="O12" s="116"/>
       <c r="P12" s="116"/>
       <c r="Q12" s="118"/>
-      <c r="R12" s="152" t="s">
+      <c r="R12" s="162" t="s">
         <v>59</v>
       </c>
       <c r="S12" s="116"/>
@@ -3796,33 +3830,33 @@
       <c r="W12" s="118"/>
     </row>
     <row r="13" spans="2:23" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B13" s="151" t="s">
+      <c r="B13" s="148" t="s">
         <v>60</v>
       </c>
       <c r="C13" s="116"/>
       <c r="D13" s="118"/>
-      <c r="E13" s="171">
+      <c r="E13" s="165">
         <f>Input_Bulanan!D11</f>
         <v>1</v>
       </c>
       <c r="F13" s="118"/>
-      <c r="G13" s="139" t="s">
+      <c r="G13" s="187" t="s">
         <v>61</v>
       </c>
       <c r="H13" s="116"/>
       <c r="I13" s="118"/>
-      <c r="J13" s="162">
+      <c r="J13" s="167">
         <f>Input_Bulanan!D8</f>
         <v>100</v>
       </c>
       <c r="K13" s="116"/>
       <c r="L13" s="118"/>
-      <c r="M13" s="157" t="s">
+      <c r="M13" s="161" t="s">
         <v>62</v>
       </c>
       <c r="N13" s="116"/>
       <c r="O13" s="118"/>
-      <c r="P13" s="161">
+      <c r="P13" s="188">
         <f>Input_Bulanan!D48</f>
         <v>5</v>
       </c>
@@ -3831,7 +3865,7 @@
         <f>Input_Bulanan!C74</f>
         <v>C1</v>
       </c>
-      <c r="S13" s="160" t="str">
+      <c r="S13" s="172" t="str">
         <f>Input_Bulanan!D74&amp;"  |  L="&amp;Input_Bulanan!F74&amp;", C="&amp;Input_Bulanan!G74&amp;", Skala="&amp;Input_Bulanan!H74&amp;" -&gt; "&amp;Input_Bulanan!I74</f>
         <v>Salt Supply Disruption (gangguan pasokan garam industri)  |  L=4, C=5, Skala=24 -&gt; High</v>
       </c>
@@ -3841,33 +3875,33 @@
       <c r="W13" s="116"/>
     </row>
     <row r="14" spans="2:23" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B14" s="151" t="s">
+      <c r="B14" s="148" t="s">
         <v>63</v>
       </c>
       <c r="C14" s="116"/>
       <c r="D14" s="118"/>
-      <c r="E14" s="171">
+      <c r="E14" s="165">
         <f>Input_Bulanan!D13</f>
         <v>1</v>
       </c>
       <c r="F14" s="118"/>
-      <c r="G14" s="139" t="s">
+      <c r="G14" s="187" t="s">
         <v>64</v>
       </c>
       <c r="H14" s="116"/>
       <c r="I14" s="118"/>
-      <c r="J14" s="162">
+      <c r="J14" s="167">
         <f>Input_Bulanan!D9</f>
         <v>100</v>
       </c>
       <c r="K14" s="116"/>
       <c r="L14" s="118"/>
-      <c r="M14" s="157" t="s">
+      <c r="M14" s="161" t="s">
         <v>65</v>
       </c>
       <c r="N14" s="116"/>
       <c r="O14" s="118"/>
-      <c r="P14" s="176">
+      <c r="P14" s="170">
         <f>Input_Bulanan!D49</f>
         <v>11</v>
       </c>
@@ -3876,7 +3910,7 @@
         <f>Input_Bulanan!C75</f>
         <v>C2</v>
       </c>
-      <c r="S14" s="160" t="str">
+      <c r="S14" s="172" t="str">
         <f>Input_Bulanan!D75&amp;"  |  L="&amp;Input_Bulanan!F75&amp;", C="&amp;Input_Bulanan!G75&amp;", Skala="&amp;Input_Bulanan!H75&amp;" -&gt; "&amp;Input_Bulanan!I75</f>
         <v>Commissioning Delay (keterlambatan commissioning)  |  L=5, C=5, Skala=25 -&gt; High</v>
       </c>
@@ -3886,33 +3920,33 @@
       <c r="W14" s="116"/>
     </row>
     <row r="15" spans="2:23" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B15" s="151" t="s">
+      <c r="B15" s="148" t="s">
         <v>66</v>
       </c>
       <c r="C15" s="116"/>
       <c r="D15" s="118"/>
-      <c r="E15" s="174">
+      <c r="E15" s="150">
         <f>Input_Bulanan!D12</f>
         <v>0</v>
       </c>
       <c r="F15" s="118"/>
-      <c r="G15" s="139" t="s">
+      <c r="G15" s="187" t="s">
         <v>67</v>
       </c>
       <c r="H15" s="116"/>
       <c r="I15" s="118"/>
-      <c r="J15" s="162">
+      <c r="J15" s="167">
         <f>Input_Bulanan!D10</f>
         <v>100</v>
       </c>
       <c r="K15" s="116"/>
       <c r="L15" s="118"/>
-      <c r="M15" s="157" t="s">
+      <c r="M15" s="161" t="s">
         <v>68</v>
       </c>
       <c r="N15" s="116"/>
       <c r="O15" s="118"/>
-      <c r="P15" s="163">
+      <c r="P15" s="189">
         <f>Input_Bulanan!D50</f>
         <v>18</v>
       </c>
@@ -3921,7 +3955,7 @@
         <f>Input_Bulanan!C76</f>
         <v>C3</v>
       </c>
-      <c r="S15" s="160" t="str">
+      <c r="S15" s="172" t="str">
         <f>Input_Bulanan!D76&amp;"  |  L="&amp;Input_Bulanan!F76&amp;", C="&amp;Input_Bulanan!G76&amp;", Skala="&amp;Input_Bulanan!H76&amp;" -&gt; "&amp;Input_Bulanan!I76</f>
         <v>EPC Interface Issue (isu EPC interface lintas kontraktor)  |  L=4, C=4, Skala=19 -&gt; Moderate to High</v>
       </c>
@@ -3931,17 +3965,17 @@
       <c r="W15" s="116"/>
     </row>
     <row r="16" spans="2:23" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B16" s="151" t="s">
+      <c r="B16" s="148" t="s">
         <v>69</v>
       </c>
       <c r="C16" s="116"/>
       <c r="D16" s="118"/>
-      <c r="E16" s="174">
+      <c r="E16" s="150">
         <f>Input_Bulanan!D14</f>
         <v>0</v>
       </c>
       <c r="F16" s="118"/>
-      <c r="G16" s="192" t="s">
+      <c r="G16" s="151" t="s">
         <v>70</v>
       </c>
       <c r="H16" s="116"/>
@@ -3949,12 +3983,12 @@
       <c r="J16" s="116"/>
       <c r="K16" s="116"/>
       <c r="L16" s="118"/>
-      <c r="M16" s="157" t="s">
+      <c r="M16" s="161" t="s">
         <v>71</v>
       </c>
       <c r="N16" s="116"/>
       <c r="O16" s="118"/>
-      <c r="P16" s="191">
+      <c r="P16" s="145">
         <f>Input_Bulanan!D51</f>
         <v>4</v>
       </c>
@@ -3963,7 +3997,7 @@
         <f>Input_Bulanan!C77</f>
         <v>C4</v>
       </c>
-      <c r="S16" s="160" t="str">
+      <c r="S16" s="172" t="str">
         <f>Input_Bulanan!D77&amp;"  |  L="&amp;Input_Bulanan!F77&amp;", C="&amp;Input_Bulanan!G77&amp;", Skala="&amp;Input_Bulanan!H77&amp;" -&gt; "&amp;Input_Bulanan!I77</f>
         <v>Long Lead Equipment (keterlambatan peralatan utama)  |  L=3, C=3, Skala=13 -&gt; Moderate</v>
       </c>
@@ -3974,12 +4008,12 @@
     </row>
     <row r="17" spans="2:23" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="L17" s="106"/>
-      <c r="M17" s="157" t="s">
+      <c r="M17" s="161" t="s">
         <v>72</v>
       </c>
       <c r="N17" s="116"/>
       <c r="O17" s="118"/>
-      <c r="P17" s="191">
+      <c r="P17" s="145">
         <f>Input_Bulanan!D52</f>
         <v>3</v>
       </c>
@@ -3991,7 +4025,7 @@
       </c>
       <c r="N18" s="103"/>
       <c r="O18" s="104"/>
-      <c r="P18" s="190">
+      <c r="P18" s="149">
         <f>Input_Bulanan!D53</f>
         <v>41</v>
       </c>
@@ -4016,20 +4050,20 @@
       <c r="Q19" s="114"/>
     </row>
     <row r="20" spans="2:23" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B20" s="177" t="s">
+      <c r="B20" s="173" t="s">
         <v>74</v>
       </c>
-      <c r="C20" s="178"/>
-      <c r="D20" s="178"/>
-      <c r="E20" s="178"/>
-      <c r="F20" s="178"/>
-      <c r="G20" s="178"/>
-      <c r="H20" s="178"/>
-      <c r="I20" s="178"/>
-      <c r="J20" s="178"/>
-      <c r="K20" s="178"/>
-      <c r="L20" s="179"/>
-      <c r="M20" s="172" t="s">
+      <c r="C20" s="174"/>
+      <c r="D20" s="174"/>
+      <c r="E20" s="174"/>
+      <c r="F20" s="174"/>
+      <c r="G20" s="174"/>
+      <c r="H20" s="174"/>
+      <c r="I20" s="174"/>
+      <c r="J20" s="174"/>
+      <c r="K20" s="174"/>
+      <c r="L20" s="175"/>
+      <c r="M20" s="186" t="s">
         <v>75</v>
       </c>
       <c r="N20" s="116"/>
@@ -4038,92 +4072,92 @@
       <c r="Q20" s="118"/>
     </row>
     <row r="21" spans="2:23" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B21" s="180"/>
-      <c r="C21" s="181"/>
-      <c r="D21" s="181"/>
-      <c r="E21" s="181"/>
-      <c r="F21" s="181"/>
-      <c r="G21" s="181"/>
-      <c r="H21" s="181"/>
-      <c r="I21" s="181"/>
-      <c r="J21" s="181"/>
-      <c r="K21" s="181"/>
-      <c r="L21" s="182"/>
-      <c r="M21" s="151" t="s">
+      <c r="B21" s="176"/>
+      <c r="C21" s="177"/>
+      <c r="D21" s="177"/>
+      <c r="E21" s="177"/>
+      <c r="F21" s="177"/>
+      <c r="G21" s="177"/>
+      <c r="H21" s="177"/>
+      <c r="I21" s="177"/>
+      <c r="J21" s="177"/>
+      <c r="K21" s="177"/>
+      <c r="L21" s="178"/>
+      <c r="M21" s="148" t="s">
         <v>76</v>
       </c>
       <c r="N21" s="116"/>
       <c r="O21" s="118"/>
-      <c r="P21" s="149">
+      <c r="P21" s="163">
         <f>Input_Bulanan!D56</f>
         <v>0.82</v>
       </c>
       <c r="Q21" s="118"/>
     </row>
     <row r="22" spans="2:23" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B22" s="180"/>
-      <c r="C22" s="181"/>
-      <c r="D22" s="181"/>
-      <c r="E22" s="181"/>
-      <c r="F22" s="181"/>
-      <c r="G22" s="181"/>
-      <c r="H22" s="181"/>
-      <c r="I22" s="181"/>
-      <c r="J22" s="181"/>
-      <c r="K22" s="181"/>
-      <c r="L22" s="182"/>
-      <c r="M22" s="151" t="s">
+      <c r="B22" s="176"/>
+      <c r="C22" s="177"/>
+      <c r="D22" s="177"/>
+      <c r="E22" s="177"/>
+      <c r="F22" s="177"/>
+      <c r="G22" s="177"/>
+      <c r="H22" s="177"/>
+      <c r="I22" s="177"/>
+      <c r="J22" s="177"/>
+      <c r="K22" s="177"/>
+      <c r="L22" s="178"/>
+      <c r="M22" s="148" t="s">
         <v>77</v>
       </c>
       <c r="N22" s="116"/>
       <c r="O22" s="118"/>
-      <c r="P22" s="149">
+      <c r="P22" s="163">
         <f>Input_Bulanan!D57</f>
         <v>0.18</v>
       </c>
       <c r="Q22" s="118"/>
     </row>
     <row r="23" spans="2:23" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B23" s="180"/>
-      <c r="C23" s="181"/>
-      <c r="D23" s="181"/>
-      <c r="E23" s="181"/>
-      <c r="F23" s="181"/>
-      <c r="G23" s="181"/>
-      <c r="H23" s="181"/>
-      <c r="I23" s="181"/>
-      <c r="J23" s="181"/>
-      <c r="K23" s="181"/>
-      <c r="L23" s="182"/>
-      <c r="M23" s="151" t="s">
+      <c r="B23" s="176"/>
+      <c r="C23" s="177"/>
+      <c r="D23" s="177"/>
+      <c r="E23" s="177"/>
+      <c r="F23" s="177"/>
+      <c r="G23" s="177"/>
+      <c r="H23" s="177"/>
+      <c r="I23" s="177"/>
+      <c r="J23" s="177"/>
+      <c r="K23" s="177"/>
+      <c r="L23" s="178"/>
+      <c r="M23" s="148" t="s">
         <v>78</v>
       </c>
       <c r="N23" s="116"/>
       <c r="O23" s="118"/>
-      <c r="P23" s="149">
+      <c r="P23" s="163">
         <f>Input_Bulanan!D58</f>
         <v>0.76</v>
       </c>
       <c r="Q23" s="118"/>
     </row>
     <row r="24" spans="2:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B24" s="183"/>
-      <c r="C24" s="184"/>
-      <c r="D24" s="184"/>
-      <c r="E24" s="184"/>
-      <c r="F24" s="184"/>
-      <c r="G24" s="184"/>
-      <c r="H24" s="184"/>
-      <c r="I24" s="184"/>
-      <c r="J24" s="184"/>
-      <c r="K24" s="184"/>
-      <c r="L24" s="185"/>
-      <c r="M24" s="151" t="s">
+      <c r="B24" s="179"/>
+      <c r="C24" s="180"/>
+      <c r="D24" s="180"/>
+      <c r="E24" s="180"/>
+      <c r="F24" s="180"/>
+      <c r="G24" s="180"/>
+      <c r="H24" s="180"/>
+      <c r="I24" s="180"/>
+      <c r="J24" s="180"/>
+      <c r="K24" s="180"/>
+      <c r="L24" s="181"/>
+      <c r="M24" s="148" t="s">
         <v>79</v>
       </c>
       <c r="N24" s="116"/>
       <c r="O24" s="118"/>
-      <c r="P24" s="168">
+      <c r="P24" s="183">
         <f>Input_Bulanan!D59</f>
         <v>5</v>
       </c>
@@ -4154,7 +4188,7 @@
       <c r="W25" s="114"/>
     </row>
     <row r="26" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B26" s="158" t="s">
+      <c r="B26" s="166" t="s">
         <v>80</v>
       </c>
       <c r="C26" s="116"/>
@@ -4180,20 +4214,20 @@
       <c r="W26" s="118"/>
     </row>
     <row r="27" spans="2:23" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B27" s="147" t="s">
+      <c r="B27" s="164" t="s">
         <v>81</v>
       </c>
       <c r="C27" s="116"/>
       <c r="D27" s="116"/>
       <c r="E27" s="116"/>
       <c r="F27" s="118"/>
-      <c r="G27" s="147" t="s">
+      <c r="G27" s="164" t="s">
         <v>82</v>
       </c>
       <c r="H27" s="116"/>
       <c r="I27" s="116"/>
       <c r="J27" s="118"/>
-      <c r="K27" s="147" t="s">
+      <c r="K27" s="164" t="s">
         <v>83</v>
       </c>
       <c r="L27" s="118"/>
@@ -4206,7 +4240,7 @@
       <c r="O27" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="P27" s="147" t="s">
+      <c r="P27" s="164" t="s">
         <v>87</v>
       </c>
       <c r="Q27" s="116"/>
@@ -4218,20 +4252,20 @@
       <c r="W27" s="118"/>
     </row>
     <row r="28" spans="2:23" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B28" s="139" t="s">
+      <c r="B28" s="187" t="s">
         <v>88</v>
       </c>
       <c r="C28" s="116"/>
       <c r="D28" s="116"/>
       <c r="E28" s="116"/>
       <c r="F28" s="118"/>
-      <c r="G28" s="150" t="s">
+      <c r="G28" s="140" t="s">
         <v>89</v>
       </c>
       <c r="H28" s="116"/>
       <c r="I28" s="116"/>
       <c r="J28" s="118"/>
-      <c r="K28" s="169">
+      <c r="K28" s="184">
         <f>Input_Bulanan!E63</f>
         <v>24</v>
       </c>
@@ -4248,7 +4282,7 @@
         <f>IF(Input_Bulanan!H63="Bahaya","V","")</f>
         <v>V</v>
       </c>
-      <c r="P28" s="189" t="s">
+      <c r="P28" s="139" t="s">
         <v>90</v>
       </c>
       <c r="Q28" s="116"/>
@@ -4260,20 +4294,20 @@
       <c r="W28" s="118"/>
     </row>
     <row r="29" spans="2:23" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B29" s="153" t="s">
+      <c r="B29" s="138" t="s">
         <v>91</v>
       </c>
       <c r="C29" s="116"/>
       <c r="D29" s="116"/>
       <c r="E29" s="116"/>
       <c r="F29" s="118"/>
-      <c r="G29" s="165" t="s">
+      <c r="G29" s="171" t="s">
         <v>92</v>
       </c>
       <c r="H29" s="116"/>
       <c r="I29" s="116"/>
       <c r="J29" s="118"/>
-      <c r="K29" s="140">
+      <c r="K29" s="146">
         <f>Input_Bulanan!E64</f>
         <v>0.73</v>
       </c>
@@ -4290,7 +4324,7 @@
         <f>IF(Input_Bulanan!H64="Bahaya","V","")</f>
         <v/>
       </c>
-      <c r="P29" s="164" t="s">
+      <c r="P29" s="169" t="s">
         <v>93</v>
       </c>
       <c r="Q29" s="116"/>
@@ -4302,20 +4336,20 @@
       <c r="W29" s="118"/>
     </row>
     <row r="30" spans="2:23" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B30" s="139" t="s">
+      <c r="B30" s="187" t="s">
         <v>94</v>
       </c>
       <c r="C30" s="116"/>
       <c r="D30" s="116"/>
       <c r="E30" s="116"/>
       <c r="F30" s="118"/>
-      <c r="G30" s="150" t="s">
+      <c r="G30" s="140" t="s">
         <v>95</v>
       </c>
       <c r="H30" s="116"/>
       <c r="I30" s="116"/>
       <c r="J30" s="118"/>
-      <c r="K30" s="170">
+      <c r="K30" s="185">
         <f>Input_Bulanan!E65</f>
         <v>0.94</v>
       </c>
@@ -4332,7 +4366,7 @@
         <f>IF(Input_Bulanan!H65="Bahaya","V","")</f>
         <v/>
       </c>
-      <c r="P30" s="189" t="s">
+      <c r="P30" s="139" t="s">
         <v>96</v>
       </c>
       <c r="Q30" s="116"/>
@@ -4344,20 +4378,20 @@
       <c r="W30" s="118"/>
     </row>
     <row r="31" spans="2:23" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B31" s="153" t="s">
+      <c r="B31" s="138" t="s">
         <v>97</v>
       </c>
       <c r="C31" s="116"/>
       <c r="D31" s="116"/>
       <c r="E31" s="116"/>
       <c r="F31" s="118"/>
-      <c r="G31" s="165" t="s">
+      <c r="G31" s="171" t="s">
         <v>98</v>
       </c>
       <c r="H31" s="116"/>
       <c r="I31" s="116"/>
       <c r="J31" s="118"/>
-      <c r="K31" s="140">
+      <c r="K31" s="146">
         <f>Input_Bulanan!E66</f>
         <v>0.75</v>
       </c>
@@ -4374,7 +4408,7 @@
         <f>IF(Input_Bulanan!H66="Bahaya","V","")</f>
         <v>V</v>
       </c>
-      <c r="P31" s="164" t="s">
+      <c r="P31" s="169" t="s">
         <v>99</v>
       </c>
       <c r="Q31" s="116"/>
@@ -4386,20 +4420,20 @@
       <c r="W31" s="118"/>
     </row>
     <row r="32" spans="2:23" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B32" s="139" t="s">
+      <c r="B32" s="187" t="s">
         <v>100</v>
       </c>
       <c r="C32" s="116"/>
       <c r="D32" s="116"/>
       <c r="E32" s="116"/>
       <c r="F32" s="118"/>
-      <c r="G32" s="150" t="s">
+      <c r="G32" s="140" t="s">
         <v>101</v>
       </c>
       <c r="H32" s="116"/>
       <c r="I32" s="116"/>
       <c r="J32" s="118"/>
-      <c r="K32" s="166">
+      <c r="K32" s="190">
         <f>Input_Bulanan!E67</f>
         <v>0.42</v>
       </c>
@@ -4416,7 +4450,7 @@
         <f>IF(Input_Bulanan!H67="Bahaya","V","")</f>
         <v>V</v>
       </c>
-      <c r="P32" s="189" t="s">
+      <c r="P32" s="139" t="s">
         <v>102</v>
       </c>
       <c r="Q32" s="116"/>
@@ -4428,20 +4462,20 @@
       <c r="W32" s="118"/>
     </row>
     <row r="33" spans="2:23" x14ac:dyDescent="0.45">
-      <c r="B33" s="153" t="s">
+      <c r="B33" s="138" t="s">
         <v>103</v>
       </c>
       <c r="C33" s="116"/>
       <c r="D33" s="116"/>
       <c r="E33" s="116"/>
       <c r="F33" s="118"/>
-      <c r="G33" s="165" t="s">
+      <c r="G33" s="171" t="s">
         <v>104</v>
       </c>
       <c r="H33" s="116"/>
       <c r="I33" s="116"/>
       <c r="J33" s="118"/>
-      <c r="K33" s="140">
+      <c r="K33" s="146">
         <f>Input_Bulanan!E68</f>
         <v>0.4</v>
       </c>
@@ -4458,7 +4492,7 @@
         <f>IF(Input_Bulanan!H68="Bahaya","V","")</f>
         <v>V</v>
       </c>
-      <c r="P33" s="164" t="s">
+      <c r="P33" s="169" t="s">
         <v>105</v>
       </c>
       <c r="Q33" s="116"/>
@@ -4494,7 +4528,7 @@
       <c r="W34" s="114"/>
     </row>
     <row r="35" spans="2:23" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B35" s="158" t="s">
+      <c r="B35" s="166" t="s">
         <v>106</v>
       </c>
       <c r="C35" s="116"/>
@@ -4520,7 +4554,7 @@
       <c r="W35" s="118"/>
     </row>
     <row r="36" spans="2:23" ht="33" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B36" s="159" t="str">
+      <c r="B36" s="154" t="str">
         <f>"Prioritas 1—2: [1] " &amp; INDEX(Risk_Action_Tracker!E$6:E$15, MATCH(LARGE(Risk_Action_Tracker!Z$6:Z$15, 1), Risk_Action_Tracker!Z$6:Z$15, 0)) &amp; " · [2] " &amp; INDEX(Risk_Action_Tracker!E$6:E$15, MATCH(LARGE(Risk_Action_Tracker!Z$6:Z$15, 2), Risk_Action_Tracker!Z$6:Z$15, 0))</f>
         <v>Prioritas 1—2: [1] Mengesahkan pembentukan tim Interface Coordinator dan menerapkan Interface Management Plan (IMP) yang mengikat seluruh kontraktor; mengharuskan Rekind menyelaraskan jadwal penyusunan gambar detail dengan kemajuan ISBL EPC-A. · [2] Memberikan dispensasi perpanjangan jaminan pelaksanaan secara terkendali; meminta Parent Company Guarantee dari PT Perusahaan Induk X (Persero) untuk menjamin ketersediaan pendanaan bila Rekind menghadapi kendala likuiditas.</v>
       </c>
@@ -4547,7 +4581,7 @@
       <c r="W36" s="118"/>
     </row>
     <row r="37" spans="2:23" ht="42.4" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B37" s="159" t="s">
+      <c r="B37" s="154" t="s">
         <v>107</v>
       </c>
       <c r="C37" s="116"/>
@@ -4574,24 +4608,70 @@
     </row>
   </sheetData>
   <mergeCells count="98">
-    <mergeCell ref="B33:F33"/>
-    <mergeCell ref="P30:W30"/>
-    <mergeCell ref="G30:J30"/>
-    <mergeCell ref="M19:Q19"/>
-    <mergeCell ref="K6:L7"/>
-    <mergeCell ref="P16:Q16"/>
-    <mergeCell ref="P32:W32"/>
-    <mergeCell ref="K31:L31"/>
-    <mergeCell ref="B29:F29"/>
-    <mergeCell ref="R5:W5"/>
-    <mergeCell ref="P28:W28"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="G28:J28"/>
-    <mergeCell ref="P18:Q18"/>
-    <mergeCell ref="P17:Q17"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="B19:L19"/>
-    <mergeCell ref="G16:L16"/>
+    <mergeCell ref="M4:W4"/>
+    <mergeCell ref="G13:I13"/>
+    <mergeCell ref="K33:L33"/>
+    <mergeCell ref="B10:F11"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="K8:L9"/>
+    <mergeCell ref="G15:I15"/>
+    <mergeCell ref="P22:Q22"/>
+    <mergeCell ref="G32:J32"/>
+    <mergeCell ref="M21:O21"/>
+    <mergeCell ref="G5:L5"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="K29:L29"/>
+    <mergeCell ref="B6:F9"/>
+    <mergeCell ref="M17:O17"/>
+    <mergeCell ref="B26:W26"/>
+    <mergeCell ref="B36:W36"/>
+    <mergeCell ref="S14:W14"/>
+    <mergeCell ref="K10:L11"/>
+    <mergeCell ref="M24:O24"/>
+    <mergeCell ref="S13:W13"/>
+    <mergeCell ref="M12:Q12"/>
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="S15:W15"/>
+    <mergeCell ref="P13:Q13"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="J13:L13"/>
+    <mergeCell ref="P15:Q15"/>
+    <mergeCell ref="P31:W31"/>
+    <mergeCell ref="G31:J31"/>
+    <mergeCell ref="K32:L32"/>
+    <mergeCell ref="B1:W1"/>
+    <mergeCell ref="P24:Q24"/>
+    <mergeCell ref="K28:L28"/>
+    <mergeCell ref="J15:L15"/>
+    <mergeCell ref="K30:L30"/>
+    <mergeCell ref="M22:O22"/>
+    <mergeCell ref="P29:W29"/>
+    <mergeCell ref="G29:J29"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="R12:W12"/>
+    <mergeCell ref="M5:Q5"/>
+    <mergeCell ref="M15:O15"/>
+    <mergeCell ref="M20:Q20"/>
+    <mergeCell ref="G14:I14"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B35:W35"/>
+    <mergeCell ref="G6:J7"/>
+    <mergeCell ref="B25:W25"/>
+    <mergeCell ref="M14:O14"/>
+    <mergeCell ref="M23:O23"/>
+    <mergeCell ref="K27:L27"/>
+    <mergeCell ref="G12:L12"/>
+    <mergeCell ref="J14:L14"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="M10:Q11"/>
+    <mergeCell ref="P33:W33"/>
+    <mergeCell ref="P14:Q14"/>
+    <mergeCell ref="G33:J33"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="S16:W16"/>
+    <mergeCell ref="B20:L24"/>
     <mergeCell ref="B2:W2"/>
     <mergeCell ref="B34:W34"/>
     <mergeCell ref="B4:L4"/>
@@ -4608,70 +4688,24 @@
     <mergeCell ref="G27:J27"/>
     <mergeCell ref="P23:Q23"/>
     <mergeCell ref="E13:F13"/>
-    <mergeCell ref="B35:W35"/>
-    <mergeCell ref="G6:J7"/>
-    <mergeCell ref="B25:W25"/>
-    <mergeCell ref="M14:O14"/>
-    <mergeCell ref="M23:O23"/>
-    <mergeCell ref="K27:L27"/>
-    <mergeCell ref="G12:L12"/>
-    <mergeCell ref="J14:L14"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="M10:Q11"/>
-    <mergeCell ref="P33:W33"/>
-    <mergeCell ref="P14:Q14"/>
-    <mergeCell ref="G33:J33"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="S16:W16"/>
-    <mergeCell ref="B20:L24"/>
-    <mergeCell ref="B1:W1"/>
-    <mergeCell ref="P24:Q24"/>
-    <mergeCell ref="K28:L28"/>
-    <mergeCell ref="J15:L15"/>
-    <mergeCell ref="K30:L30"/>
-    <mergeCell ref="M22:O22"/>
-    <mergeCell ref="P29:W29"/>
-    <mergeCell ref="G29:J29"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="R12:W12"/>
-    <mergeCell ref="M5:Q5"/>
-    <mergeCell ref="M15:O15"/>
-    <mergeCell ref="M20:Q20"/>
-    <mergeCell ref="G14:I14"/>
-    <mergeCell ref="B5:F5"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="B36:W36"/>
-    <mergeCell ref="S14:W14"/>
-    <mergeCell ref="K10:L11"/>
-    <mergeCell ref="M24:O24"/>
-    <mergeCell ref="S13:W13"/>
-    <mergeCell ref="M12:Q12"/>
-    <mergeCell ref="B32:F32"/>
-    <mergeCell ref="B28:F28"/>
-    <mergeCell ref="S15:W15"/>
-    <mergeCell ref="P13:Q13"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="J13:L13"/>
-    <mergeCell ref="P15:Q15"/>
-    <mergeCell ref="P31:W31"/>
-    <mergeCell ref="G31:J31"/>
-    <mergeCell ref="K32:L32"/>
-    <mergeCell ref="M4:W4"/>
-    <mergeCell ref="G13:I13"/>
-    <mergeCell ref="K33:L33"/>
-    <mergeCell ref="B10:F11"/>
-    <mergeCell ref="B27:F27"/>
-    <mergeCell ref="K8:L9"/>
-    <mergeCell ref="G15:I15"/>
-    <mergeCell ref="P22:Q22"/>
-    <mergeCell ref="G32:J32"/>
-    <mergeCell ref="M21:O21"/>
-    <mergeCell ref="G5:L5"/>
-    <mergeCell ref="B31:F31"/>
-    <mergeCell ref="K29:L29"/>
-    <mergeCell ref="B6:F9"/>
-    <mergeCell ref="M17:O17"/>
-    <mergeCell ref="B26:W26"/>
+    <mergeCell ref="R5:W5"/>
+    <mergeCell ref="P28:W28"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="G28:J28"/>
+    <mergeCell ref="P18:Q18"/>
+    <mergeCell ref="P17:Q17"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="B19:L19"/>
+    <mergeCell ref="G16:L16"/>
+    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="P30:W30"/>
+    <mergeCell ref="G30:J30"/>
+    <mergeCell ref="M19:Q19"/>
+    <mergeCell ref="K6:L7"/>
+    <mergeCell ref="P16:Q16"/>
+    <mergeCell ref="P32:W32"/>
+    <mergeCell ref="K31:L31"/>
+    <mergeCell ref="B29:F29"/>
   </mergeCells>
   <conditionalFormatting sqref="B10:F11">
     <cfRule type="expression" dxfId="11" priority="2">
@@ -4750,7 +4784,7 @@
       <c r="E2" s="13"/>
     </row>
     <row r="3" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="133" t="s">
+      <c r="A3" s="125" t="s">
         <v>384</v>
       </c>
       <c r="B3" s="114"/>
@@ -4759,7 +4793,7 @@
       <c r="E3" s="114"/>
     </row>
     <row r="5" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="117" t="s">
+      <c r="A5" s="120" t="s">
         <v>109</v>
       </c>
       <c r="B5" s="116"/>
@@ -4878,7 +4912,7 @@
       </c>
     </row>
     <row r="14" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A14" s="137" t="s">
+      <c r="A14" s="113" t="s">
         <v>130</v>
       </c>
       <c r="B14" s="114"/>
@@ -4887,7 +4921,7 @@
       <c r="E14" s="114"/>
     </row>
     <row r="15" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="113" t="s">
+      <c r="A15" s="134" t="s">
         <v>131</v>
       </c>
       <c r="B15" s="114"/>
@@ -4896,7 +4930,7 @@
       <c r="E15" s="114"/>
     </row>
     <row r="17" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="117" t="s">
+      <c r="A17" s="120" t="s">
         <v>132</v>
       </c>
       <c r="B17" s="116"/>
@@ -4911,7 +4945,7 @@
       <c r="B18" s="14" t="s">
         <v>133</v>
       </c>
-      <c r="C18" s="135" t="s">
+      <c r="C18" s="122" t="s">
         <v>134</v>
       </c>
       <c r="D18" s="116"/>
@@ -4924,7 +4958,7 @@
       <c r="B19" s="110">
         <v>0.25</v>
       </c>
-      <c r="C19" s="122" t="s">
+      <c r="C19" s="123" t="s">
         <v>136</v>
       </c>
       <c r="D19" s="116"/>
@@ -4950,7 +4984,7 @@
       <c r="B21" s="110">
         <v>0.2</v>
       </c>
-      <c r="C21" s="122" t="s">
+      <c r="C21" s="123" t="s">
         <v>140</v>
       </c>
       <c r="D21" s="116"/>
@@ -4976,14 +5010,14 @@
       <c r="B23" s="110">
         <v>0.15</v>
       </c>
-      <c r="C23" s="122" t="s">
+      <c r="C23" s="123" t="s">
         <v>144</v>
       </c>
       <c r="D23" s="116"/>
       <c r="E23" s="116"/>
     </row>
     <row r="25" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A25" s="117" t="s">
+      <c r="A25" s="120" t="s">
         <v>145</v>
       </c>
       <c r="B25" s="116"/>
@@ -4998,7 +5032,7 @@
       <c r="B26" s="14" t="s">
         <v>133</v>
       </c>
-      <c r="C26" s="135" t="s">
+      <c r="C26" s="122" t="s">
         <v>134</v>
       </c>
       <c r="D26" s="116"/>
@@ -5011,7 +5045,7 @@
       <c r="B27" s="110">
         <v>0.25</v>
       </c>
-      <c r="C27" s="122" t="s">
+      <c r="C27" s="123" t="s">
         <v>147</v>
       </c>
       <c r="D27" s="116"/>
@@ -5037,7 +5071,7 @@
       <c r="B29" s="110">
         <v>0.35</v>
       </c>
-      <c r="C29" s="122" t="s">
+      <c r="C29" s="123" t="s">
         <v>151</v>
       </c>
       <c r="D29" s="116"/>
@@ -5057,7 +5091,7 @@
       <c r="E30" s="116"/>
     </row>
     <row r="32" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A32" s="117" t="s">
+      <c r="A32" s="120" t="s">
         <v>154</v>
       </c>
       <c r="B32" s="116"/>
@@ -5072,7 +5106,7 @@
       <c r="B33" s="14" t="s">
         <v>133</v>
       </c>
-      <c r="C33" s="135" t="s">
+      <c r="C33" s="122" t="s">
         <v>134</v>
       </c>
       <c r="D33" s="116"/>
@@ -5098,7 +5132,7 @@
       <c r="B35" s="110">
         <v>0.2</v>
       </c>
-      <c r="C35" s="122" t="s">
+      <c r="C35" s="123" t="s">
         <v>158</v>
       </c>
       <c r="D35" s="116"/>
@@ -5124,7 +5158,7 @@
       <c r="B37" s="110">
         <v>0.2</v>
       </c>
-      <c r="C37" s="122" t="s">
+      <c r="C37" s="123" t="s">
         <v>162</v>
       </c>
       <c r="D37" s="116"/>
@@ -5144,7 +5178,7 @@
       <c r="E38" s="116"/>
     </row>
     <row r="40" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A40" s="117" t="s">
+      <c r="A40" s="120" t="s">
         <v>165</v>
       </c>
       <c r="B40" s="116"/>
@@ -5293,7 +5327,7 @@
       </c>
     </row>
     <row r="49" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A49" s="117" t="s">
+      <c r="A49" s="120" t="s">
         <v>202</v>
       </c>
       <c r="B49" s="116"/>
@@ -5302,7 +5336,7 @@
       <c r="E49" s="118"/>
     </row>
     <row r="50" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A50" s="134" t="s">
+      <c r="A50" s="129" t="s">
         <v>385</v>
       </c>
       <c r="B50" s="114"/>
@@ -5317,7 +5351,7 @@
       <c r="B51" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="C51" s="121" t="s">
+      <c r="C51" s="117" t="s">
         <v>204</v>
       </c>
       <c r="D51" s="116"/>
@@ -5330,7 +5364,7 @@
       <c r="B52" s="30" t="s">
         <v>205</v>
       </c>
-      <c r="C52" s="120" t="s">
+      <c r="C52" s="121" t="s">
         <v>206</v>
       </c>
       <c r="D52" s="116"/>
@@ -5343,7 +5377,7 @@
       <c r="B53" s="32" t="s">
         <v>207</v>
       </c>
-      <c r="C53" s="127" t="s">
+      <c r="C53" s="119" t="s">
         <v>208</v>
       </c>
       <c r="D53" s="116"/>
@@ -5356,7 +5390,7 @@
       <c r="B54" s="30" t="s">
         <v>209</v>
       </c>
-      <c r="C54" s="120" t="s">
+      <c r="C54" s="121" t="s">
         <v>210</v>
       </c>
       <c r="D54" s="116"/>
@@ -5369,7 +5403,7 @@
       <c r="B55" s="32" t="s">
         <v>211</v>
       </c>
-      <c r="C55" s="127" t="s">
+      <c r="C55" s="119" t="s">
         <v>212</v>
       </c>
       <c r="D55" s="116"/>
@@ -5382,14 +5416,14 @@
       <c r="B56" s="30" t="s">
         <v>213</v>
       </c>
-      <c r="C56" s="120" t="s">
+      <c r="C56" s="121" t="s">
         <v>214</v>
       </c>
       <c r="D56" s="116"/>
       <c r="E56" s="116"/>
     </row>
     <row r="58" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A58" s="117" t="s">
+      <c r="A58" s="120" t="s">
         <v>215</v>
       </c>
       <c r="B58" s="116"/>
@@ -5404,7 +5438,7 @@
       <c r="B59" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="C59" s="121" t="s">
+      <c r="C59" s="117" t="s">
         <v>217</v>
       </c>
       <c r="D59" s="116"/>
@@ -5417,7 +5451,7 @@
       <c r="B60" s="30" t="s">
         <v>218</v>
       </c>
-      <c r="C60" s="120" t="s">
+      <c r="C60" s="121" t="s">
         <v>219</v>
       </c>
       <c r="D60" s="116"/>
@@ -5430,7 +5464,7 @@
       <c r="B61" s="32" t="s">
         <v>220</v>
       </c>
-      <c r="C61" s="127" t="s">
+      <c r="C61" s="119" t="s">
         <v>221</v>
       </c>
       <c r="D61" s="116"/>
@@ -5443,7 +5477,7 @@
       <c r="B62" s="30" t="s">
         <v>222</v>
       </c>
-      <c r="C62" s="120" t="s">
+      <c r="C62" s="121" t="s">
         <v>223</v>
       </c>
       <c r="D62" s="116"/>
@@ -5456,7 +5490,7 @@
       <c r="B63" s="32" t="s">
         <v>224</v>
       </c>
-      <c r="C63" s="127" t="s">
+      <c r="C63" s="119" t="s">
         <v>225</v>
       </c>
       <c r="D63" s="116"/>
@@ -5469,14 +5503,14 @@
       <c r="B64" s="30" t="s">
         <v>226</v>
       </c>
-      <c r="C64" s="120" t="s">
+      <c r="C64" s="121" t="s">
         <v>227</v>
       </c>
       <c r="D64" s="116"/>
       <c r="E64" s="116"/>
     </row>
     <row r="66" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A66" s="117" t="s">
+      <c r="A66" s="120" t="s">
         <v>386</v>
       </c>
       <c r="B66" s="116"/>
@@ -5485,7 +5519,7 @@
       <c r="E66" s="118"/>
     </row>
     <row r="67" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A67" s="136" t="s">
+      <c r="A67" s="130" t="s">
         <v>228</v>
       </c>
       <c r="B67" s="114"/>
@@ -5500,7 +5534,7 @@
       <c r="B68" s="9" t="s">
         <v>230</v>
       </c>
-      <c r="C68" s="121" t="s">
+      <c r="C68" s="117" t="s">
         <v>231</v>
       </c>
       <c r="D68" s="116"/>
@@ -5513,7 +5547,7 @@
       <c r="B69" s="37" t="s">
         <v>232</v>
       </c>
-      <c r="C69" s="125" t="s">
+      <c r="C69" s="124" t="s">
         <v>233</v>
       </c>
       <c r="D69" s="116"/>
@@ -5526,7 +5560,7 @@
       <c r="B70" s="37" t="s">
         <v>234</v>
       </c>
-      <c r="C70" s="125" t="s">
+      <c r="C70" s="124" t="s">
         <v>235</v>
       </c>
       <c r="D70" s="116"/>
@@ -5539,7 +5573,7 @@
       <c r="B71" s="37" t="s">
         <v>236</v>
       </c>
-      <c r="C71" s="125" t="s">
+      <c r="C71" s="124" t="s">
         <v>237</v>
       </c>
       <c r="D71" s="116"/>
@@ -5552,7 +5586,7 @@
       <c r="B72" s="37" t="s">
         <v>238</v>
       </c>
-      <c r="C72" s="125" t="s">
+      <c r="C72" s="124" t="s">
         <v>239</v>
       </c>
       <c r="D72" s="116"/>
@@ -5565,14 +5599,14 @@
       <c r="B73" s="37" t="s">
         <v>240</v>
       </c>
-      <c r="C73" s="125" t="s">
+      <c r="C73" s="124" t="s">
         <v>241</v>
       </c>
       <c r="D73" s="116"/>
       <c r="E73" s="116"/>
     </row>
     <row r="75" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A75" s="117" t="s">
+      <c r="A75" s="120" t="s">
         <v>242</v>
       </c>
       <c r="B75" s="116"/>
@@ -5587,7 +5621,7 @@
       <c r="B76" s="111">
         <v>0.4</v>
       </c>
-      <c r="C76" s="120" t="s">
+      <c r="C76" s="121" t="s">
         <v>244</v>
       </c>
       <c r="D76" s="116"/>
@@ -5600,7 +5634,7 @@
       <c r="B77" s="110">
         <v>0.4</v>
       </c>
-      <c r="C77" s="127" t="s">
+      <c r="C77" s="119" t="s">
         <v>246</v>
       </c>
       <c r="D77" s="116"/>
@@ -5613,14 +5647,14 @@
       <c r="B78" s="111">
         <v>0.2</v>
       </c>
-      <c r="C78" s="120" t="s">
+      <c r="C78" s="121" t="s">
         <v>382</v>
       </c>
       <c r="D78" s="116"/>
       <c r="E78" s="116"/>
     </row>
     <row r="79" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A79" s="123" t="s">
+      <c r="A79" s="136" t="s">
         <v>248</v>
       </c>
       <c r="B79" s="114"/>
@@ -5647,7 +5681,7 @@
       <c r="F86" s="44"/>
     </row>
     <row r="87" spans="1:6" ht="43.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A87" s="126" t="s">
+      <c r="A87" s="131" t="s">
         <v>388</v>
       </c>
       <c r="B87" s="114"/>
@@ -6177,7 +6211,7 @@
       </c>
     </row>
     <row r="116" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A116" s="126" t="s">
+      <c r="A116" s="131" t="s">
         <v>389</v>
       </c>
       <c r="B116" s="114"/>
@@ -6197,7 +6231,7 @@
       <c r="F118" s="44"/>
     </row>
     <row r="119" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A119" s="126" t="s">
+      <c r="A119" s="131" t="s">
         <v>261</v>
       </c>
       <c r="B119" s="114"/>
@@ -6210,7 +6244,7 @@
       <c r="A121" s="51" t="s">
         <v>262</v>
       </c>
-      <c r="B121" s="129" t="s">
+      <c r="B121" s="133" t="s">
         <v>263</v>
       </c>
       <c r="C121" s="114"/>
@@ -6223,33 +6257,33 @@
       <c r="A122" s="52" t="s">
         <v>84</v>
       </c>
-      <c r="B122" s="130" t="s">
+      <c r="B122" s="126" t="s">
         <v>265</v>
       </c>
-      <c r="C122" s="131"/>
-      <c r="D122" s="132"/>
+      <c r="C122" s="127"/>
+      <c r="D122" s="128"/>
       <c r="E122" s="53"/>
     </row>
     <row r="123" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A123" s="54" t="s">
         <v>85</v>
       </c>
-      <c r="B123" s="130" t="s">
+      <c r="B123" s="126" t="s">
         <v>266</v>
       </c>
-      <c r="C123" s="131"/>
-      <c r="D123" s="132"/>
+      <c r="C123" s="127"/>
+      <c r="D123" s="128"/>
       <c r="E123" s="53"/>
     </row>
     <row r="124" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A124" s="55" t="s">
         <v>86</v>
       </c>
-      <c r="B124" s="130" t="s">
+      <c r="B124" s="126" t="s">
         <v>267</v>
       </c>
-      <c r="C124" s="131"/>
-      <c r="D124" s="132"/>
+      <c r="C124" s="127"/>
+      <c r="D124" s="128"/>
       <c r="E124" s="53"/>
     </row>
     <row r="127" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -6263,7 +6297,7 @@
       <c r="F127" s="94"/>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A129" s="124" t="s">
+      <c r="A129" s="137" t="s">
         <v>269</v>
       </c>
       <c r="B129" s="114"/>
@@ -6353,7 +6387,7 @@
       </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A136" s="119" t="s">
+      <c r="A136" s="135" t="s">
         <v>288</v>
       </c>
       <c r="B136" s="114"/>
@@ -6373,7 +6407,7 @@
       <c r="F139" s="94"/>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A141" s="128" t="s">
+      <c r="A141" s="132" t="s">
         <v>391</v>
       </c>
       <c r="B141" s="114"/>
@@ -6450,6 +6484,53 @@
     </row>
   </sheetData>
   <mergeCells count="63">
+    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="A49:E49"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A136:F136"/>
+    <mergeCell ref="C56:E56"/>
+    <mergeCell ref="C59:E59"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="A79:E79"/>
+    <mergeCell ref="C51:E51"/>
+    <mergeCell ref="A129:F129"/>
+    <mergeCell ref="C60:E60"/>
+    <mergeCell ref="C36:E36"/>
+    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="C76:E76"/>
+    <mergeCell ref="C71:E71"/>
+    <mergeCell ref="C52:E52"/>
+    <mergeCell ref="A116:F116"/>
+    <mergeCell ref="C61:E61"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="A141:F141"/>
+    <mergeCell ref="C70:E70"/>
+    <mergeCell ref="A75:E75"/>
+    <mergeCell ref="A66:E66"/>
+    <mergeCell ref="B121:D121"/>
+    <mergeCell ref="B122:D122"/>
+    <mergeCell ref="A119:F119"/>
+    <mergeCell ref="A58:E58"/>
+    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="A87:F87"/>
+    <mergeCell ref="C63:E63"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="C38:E38"/>
+    <mergeCell ref="B124:D124"/>
+    <mergeCell ref="C72:E72"/>
+    <mergeCell ref="A50:E50"/>
+    <mergeCell ref="C28:E28"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="C37:E37"/>
+    <mergeCell ref="C53:E53"/>
+    <mergeCell ref="B123:D123"/>
+    <mergeCell ref="C69:E69"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="C78:E78"/>
+    <mergeCell ref="A32:E32"/>
+    <mergeCell ref="A67:E67"/>
     <mergeCell ref="A14:E14"/>
     <mergeCell ref="C30:E30"/>
     <mergeCell ref="C68:E68"/>
@@ -6466,53 +6547,6 @@
     <mergeCell ref="A40:E40"/>
     <mergeCell ref="C73:E73"/>
     <mergeCell ref="C64:E64"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="C38:E38"/>
-    <mergeCell ref="B124:D124"/>
-    <mergeCell ref="C72:E72"/>
-    <mergeCell ref="A50:E50"/>
-    <mergeCell ref="C28:E28"/>
-    <mergeCell ref="C19:E19"/>
-    <mergeCell ref="C37:E37"/>
-    <mergeCell ref="C53:E53"/>
-    <mergeCell ref="B123:D123"/>
-    <mergeCell ref="C69:E69"/>
-    <mergeCell ref="C18:E18"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="C78:E78"/>
-    <mergeCell ref="A32:E32"/>
-    <mergeCell ref="A67:E67"/>
-    <mergeCell ref="C52:E52"/>
-    <mergeCell ref="A116:F116"/>
-    <mergeCell ref="C61:E61"/>
-    <mergeCell ref="C23:E23"/>
-    <mergeCell ref="A141:F141"/>
-    <mergeCell ref="C70:E70"/>
-    <mergeCell ref="A75:E75"/>
-    <mergeCell ref="A66:E66"/>
-    <mergeCell ref="B121:D121"/>
-    <mergeCell ref="B122:D122"/>
-    <mergeCell ref="A119:F119"/>
-    <mergeCell ref="A58:E58"/>
-    <mergeCell ref="C35:E35"/>
-    <mergeCell ref="A87:F87"/>
-    <mergeCell ref="C63:E63"/>
-    <mergeCell ref="A15:E15"/>
-    <mergeCell ref="C22:E22"/>
-    <mergeCell ref="A49:E49"/>
-    <mergeCell ref="A25:E25"/>
-    <mergeCell ref="A136:F136"/>
-    <mergeCell ref="C56:E56"/>
-    <mergeCell ref="C59:E59"/>
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="A79:E79"/>
-    <mergeCell ref="C51:E51"/>
-    <mergeCell ref="A129:F129"/>
-    <mergeCell ref="C60:E60"/>
-    <mergeCell ref="C36:E36"/>
-    <mergeCell ref="C27:E27"/>
-    <mergeCell ref="C76:E76"/>
-    <mergeCell ref="C71:E71"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -6547,13 +6581,27 @@
       </c>
     </row>
     <row r="3" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C3" s="133" t="s">
+      <c r="C3" s="125" t="s">
         <v>302</v>
       </c>
       <c r="D3" s="114"/>
       <c r="E3" s="114"/>
       <c r="F3" s="114"/>
       <c r="G3" s="114"/>
+    </row>
+    <row r="4" spans="3:7" x14ac:dyDescent="0.45">
+      <c r="C4" s="198" t="s">
+        <v>408</v>
+      </c>
+      <c r="D4" s="199" t="s">
+        <v>409</v>
+      </c>
+      <c r="F4" s="198" t="s">
+        <v>410</v>
+      </c>
+      <c r="G4" s="199" t="s">
+        <v>411</v>
+      </c>
     </row>
     <row r="5" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C5" s="56" t="s">
@@ -7397,7 +7445,7 @@
       <c r="G2" s="114"/>
     </row>
     <row r="3" spans="2:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B3" s="133" t="s">
+      <c r="B3" s="125" t="s">
         <v>394</v>
       </c>
       <c r="C3" s="114"/>

</xml_diff>

<commit_message>
Menambahkan Regulatory Readiness ke CRI dan memperbaiki formatting Date untuk First Shipment
</commit_message>
<xml_diff>
--- a/Template_Dashboard_v2.xlsx
+++ b/Template_Dashboard_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://365mic-my.sharepoint.com/personal/ipanjez_365mic_onmicrosoft_com/Documents/Learn/Coding/Dashboard Proyek Soda Ash/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="161" documentId="11_FBD64D39D349D756657D4B1399D967C19B799422" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{481309FE-C72E-4AFB-856F-AD91A3A88ACE}"/>
+  <xr:revisionPtr revIDLastSave="172" documentId="11_FBD64D39D349D756657D4B1399D967C19B799422" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EBAE5EFE-B06E-4D8A-B1E3-4916D244B9BB}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -473,7 +473,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C66" authorId="1" shapeId="0" xr:uid="{C20A8778-28FA-465F-A8ED-DDA081087E76}">
+    <comment ref="C67" authorId="1" shapeId="0" xr:uid="{C20A8778-28FA-465F-A8ED-DDA081087E76}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -481,7 +481,7 @@
     First Shipment, Delay dengan tolerance (On Time, sudah Waspada)</t>
       </text>
     </comment>
-    <comment ref="C67" authorId="2" shapeId="0" xr:uid="{18281803-C38B-4547-B84B-0772199CD57F}">
+    <comment ref="C68" authorId="2" shapeId="0" xr:uid="{18281803-C38B-4547-B84B-0772199CD57F}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -489,7 +489,7 @@
     Project Progress</t>
       </text>
     </comment>
-    <comment ref="C68" authorId="3" shapeId="0" xr:uid="{8AC54FF4-8EEE-43E7-86D8-9BC271053192}">
+    <comment ref="C69" authorId="3" shapeId="0" xr:uid="{8AC54FF4-8EEE-43E7-86D8-9BC271053192}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -502,7 +502,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="527" uniqueCount="418">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="419">
   <si>
     <t>EXECUTIVE ACTION TRACKER — DIREKSI / PROJECT STEERING COMMITTEE (PSC)</t>
   </si>
@@ -1477,21 +1477,9 @@
     <t>4. COMMERCIAL READINESS INDEX (CRI) — skor kesiapan tiap parameter</t>
   </si>
   <si>
-    <t>Offtake Agreement (bobot 20%)</t>
-  </si>
-  <si>
-    <t>Marketing Strategy (bobot 20%)</t>
-  </si>
-  <si>
     <t>Distribution Readiness (bobot 15%)</t>
   </si>
   <si>
-    <t>Operation Team Ready (bobot 20%)</t>
-  </si>
-  <si>
-    <t>Product Qualification (bobot 25%)</t>
-  </si>
-  <si>
     <t>CRI — Commercial Readiness Index (tertimbang)</t>
   </si>
   <si>
@@ -1760,15 +1748,31 @@
   </si>
   <si>
     <t>Offtaker Agreement</t>
+  </si>
+  <si>
+    <t>Offtake Agreement (bobot 15%)</t>
+  </si>
+  <si>
+    <t>Marketing Strategy (bobot 15%)</t>
+  </si>
+  <si>
+    <t>Operation Team Ready (bobot 15%)</t>
+  </si>
+  <si>
+    <t>Product Qualification (bobot 20%)</t>
+  </si>
+  <si>
+    <t>Regulatory Readiness (bobot 20%)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
     <numFmt numFmtId="165" formatCode="#,##0.0;\(#,##0.0\)"/>
+    <numFmt numFmtId="166" formatCode="dd\-mmm\-yy"/>
   </numFmts>
   <fonts count="54" x14ac:knownFonts="1">
     <font>
@@ -2508,7 +2512,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="200">
+  <cellXfs count="202">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -2806,207 +2810,207 @@
     <xf numFmtId="0" fontId="51" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="52" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="53" fillId="30" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="28" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="8" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="1" fontId="18" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="24" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="18" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="17" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="15" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="18" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="23" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="24" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="24" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="24" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="18" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="18" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="24" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="8" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="17" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="10" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="24" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="23" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="24" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="24" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="15" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="37" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -3018,6 +3022,12 @@
     <xf numFmtId="0" fontId="39" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="36" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3394,13 +3404,13 @@
 
 <file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="C66" dT="2026-07-17T01:48:15.15" personId="{636F4FD5-16A3-4E69-B58D-B92F078D64D6}" id="{C20A8778-28FA-465F-A8ED-DDA081087E76}">
+  <threadedComment ref="C67" dT="2026-07-17T01:48:15.15" personId="{636F4FD5-16A3-4E69-B58D-B92F078D64D6}" id="{C20A8778-28FA-465F-A8ED-DDA081087E76}">
     <text>First Shipment, Delay dengan tolerance (On Time, sudah Waspada)</text>
   </threadedComment>
-  <threadedComment ref="C67" dT="2026-07-17T01:47:50.28" personId="{636F4FD5-16A3-4E69-B58D-B92F078D64D6}" id="{18281803-C38B-4547-B84B-0772199CD57F}">
+  <threadedComment ref="C68" dT="2026-07-17T01:47:50.28" personId="{636F4FD5-16A3-4E69-B58D-B92F078D64D6}" id="{18281803-C38B-4547-B84B-0772199CD57F}">
     <text>Project Progress</text>
   </threadedComment>
-  <threadedComment ref="C68" dT="2026-07-17T01:48:49.17" personId="{636F4FD5-16A3-4E69-B58D-B92F078D64D6}" id="{8AC54FF4-8EEE-43E7-86D8-9BC271053192}">
+  <threadedComment ref="C69" dT="2026-07-17T01:48:49.17" personId="{636F4FD5-16A3-4E69-B58D-B92F078D64D6}" id="{8AC54FF4-8EEE-43E7-86D8-9BC271053192}">
     <text>Offtaker Agreement</text>
   </threadedComment>
 </ThreadedComments>
@@ -3422,8 +3432,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:23" ht="30" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B1" s="169" t="s">
-        <v>368</v>
+      <c r="B1" s="184" t="s">
+        <v>364</v>
       </c>
       <c r="C1" s="118"/>
       <c r="D1" s="118"/>
@@ -3448,7 +3458,7 @@
       <c r="W1" s="120"/>
     </row>
     <row r="2" spans="2:23" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B2" s="188" t="str">
+      <c r="B2" s="154" t="str">
         <f ca="1">"Reporting Period: "&amp;Input_Bulanan!D5&amp;"   |   Status: "&amp;Input_Bulanan!F5&amp;"   |   Dicetak: "&amp;TEXT(TODAY(),"DD-MM-YYYY")</f>
         <v>Reporting Period: Agustus 2026   |   Status: DRAFT   |   Dicetak: 20-07-2026</v>
       </c>
@@ -3476,7 +3486,7 @@
     </row>
     <row r="3" spans="2:23" ht="6" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="4" spans="2:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B4" s="140" t="s">
+      <c r="B4" s="155" t="s">
         <v>47</v>
       </c>
       <c r="C4" s="118"/>
@@ -3489,7 +3499,7 @@
       <c r="J4" s="118"/>
       <c r="K4" s="118"/>
       <c r="L4" s="120"/>
-      <c r="M4" s="140" t="s">
+      <c r="M4" s="155" t="s">
         <v>48</v>
       </c>
       <c r="N4" s="118"/>
@@ -3504,14 +3514,14 @@
       <c r="W4" s="120"/>
     </row>
     <row r="5" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B5" s="154" t="s">
+      <c r="B5" s="164" t="s">
         <v>49</v>
       </c>
       <c r="C5" s="118"/>
       <c r="D5" s="118"/>
       <c r="E5" s="118"/>
       <c r="F5" s="120"/>
-      <c r="G5" s="154" t="s">
+      <c r="G5" s="164" t="s">
         <v>50</v>
       </c>
       <c r="H5" s="118"/>
@@ -3519,14 +3529,14 @@
       <c r="J5" s="118"/>
       <c r="K5" s="118"/>
       <c r="L5" s="120"/>
-      <c r="M5" s="154" t="s">
+      <c r="M5" s="164" t="s">
         <v>51</v>
       </c>
       <c r="N5" s="118"/>
       <c r="O5" s="118"/>
       <c r="P5" s="118"/>
       <c r="Q5" s="120"/>
-      <c r="R5" s="190" t="s">
+      <c r="R5" s="149" t="s">
         <v>52</v>
       </c>
       <c r="S5" s="118"/>
@@ -3536,256 +3546,256 @@
       <c r="W5" s="120"/>
     </row>
     <row r="6" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B6" s="156">
-        <f>((IF(Input_Bulanan!D12&gt;=1,100,Input_Bulanan!D12*100)*0.2)+(IF(Input_Bulanan!D14&gt;=1,100,Input_Bulanan!D14*100)*0.2)+(Input_Bulanan!D24*100*0.2)+(Input_Bulanan!D32*100*0.2)+(Input_Bulanan!D41*100*0.2))/100</f>
-        <v>0.70820000000000005</v>
-      </c>
-      <c r="C6" s="144"/>
-      <c r="D6" s="144"/>
-      <c r="E6" s="144"/>
-      <c r="F6" s="145"/>
-      <c r="G6" s="175" t="s">
+      <c r="B6" s="194">
+        <f>((IF(Input_Bulanan!D12&gt;=1,100,Input_Bulanan!D12*100)*0.2)+(IF(Input_Bulanan!D14&gt;=1,100,Input_Bulanan!D14*100)*0.2)+(Input_Bulanan!D24*100*0.2)+(Input_Bulanan!D32*100*0.2)+(Input_Bulanan!D42*100*0.2))/100</f>
+        <v>0.70420000000000005</v>
+      </c>
+      <c r="C6" s="158"/>
+      <c r="D6" s="158"/>
+      <c r="E6" s="158"/>
+      <c r="F6" s="144"/>
+      <c r="G6" s="162" t="s">
         <v>53</v>
       </c>
-      <c r="H6" s="144"/>
-      <c r="I6" s="144"/>
-      <c r="J6" s="144"/>
-      <c r="K6" s="150">
+      <c r="H6" s="158"/>
+      <c r="I6" s="158"/>
+      <c r="J6" s="158"/>
+      <c r="K6" s="143">
         <f>Input_Bulanan!D24</f>
         <v>0.21450000000000002</v>
       </c>
-      <c r="L6" s="145"/>
-      <c r="M6" s="189" t="str">
-        <f>Input_Bulanan!D48</f>
+      <c r="L6" s="144"/>
+      <c r="M6" s="157" t="str">
+        <f>Input_Bulanan!D49</f>
         <v>Moderate</v>
       </c>
-      <c r="N6" s="144"/>
-      <c r="O6" s="144"/>
-      <c r="P6" s="144"/>
-      <c r="Q6" s="145"/>
+      <c r="N6" s="158"/>
+      <c r="O6" s="158"/>
+      <c r="P6" s="158"/>
+      <c r="Q6" s="144"/>
       <c r="R6" s="1" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
       <c r="S6" s="5" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=1,Input_Bulanan!$F$74=5),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=1,Input_Bulanan!$F$75=5),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=1,Input_Bulanan!$F$76=5),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=1,Input_Bulanan!$F$77=5),Input_Bulanan!$C$77,""))))</f>
+        <f>IF(AND(Input_Bulanan!$G$75=1,Input_Bulanan!$F$75=5),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=1,Input_Bulanan!$F$76=5),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=1,Input_Bulanan!$F$77=5),Input_Bulanan!$C$77,IF(AND(Input_Bulanan!$G$78=1,Input_Bulanan!$F$78=5),Input_Bulanan!$C$78,""))))</f>
         <v/>
       </c>
       <c r="T6" s="3" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=2,Input_Bulanan!$F$74=5),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=2,Input_Bulanan!$F$75=5),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=2,Input_Bulanan!$F$76=5),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=2,Input_Bulanan!$F$77=5),Input_Bulanan!$C$77,""))))</f>
+        <f>IF(AND(Input_Bulanan!$G$75=2,Input_Bulanan!$F$75=5),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=2,Input_Bulanan!$F$76=5),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=2,Input_Bulanan!$F$77=5),Input_Bulanan!$C$77,IF(AND(Input_Bulanan!$G$78=2,Input_Bulanan!$F$78=5),Input_Bulanan!$C$78,""))))</f>
         <v/>
       </c>
       <c r="U6" s="4" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=3,Input_Bulanan!$F$74=5),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=3,Input_Bulanan!$F$75=5),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=3,Input_Bulanan!$F$76=5),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=3,Input_Bulanan!$F$77=5),Input_Bulanan!$C$77,""))))</f>
+        <f>IF(AND(Input_Bulanan!$G$75=3,Input_Bulanan!$F$75=5),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=3,Input_Bulanan!$F$76=5),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=3,Input_Bulanan!$F$77=5),Input_Bulanan!$C$77,IF(AND(Input_Bulanan!$G$78=3,Input_Bulanan!$F$78=5),Input_Bulanan!$C$78,""))))</f>
         <v/>
       </c>
       <c r="V6" s="2" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=4,Input_Bulanan!$F$74=5),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=4,Input_Bulanan!$F$75=5),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=4,Input_Bulanan!$F$76=5),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=4,Input_Bulanan!$F$77=5),Input_Bulanan!$C$77,""))))</f>
+        <f>IF(AND(Input_Bulanan!$G$75=4,Input_Bulanan!$F$75=5),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=4,Input_Bulanan!$F$76=5),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=4,Input_Bulanan!$F$77=5),Input_Bulanan!$C$77,IF(AND(Input_Bulanan!$G$78=4,Input_Bulanan!$F$78=5),Input_Bulanan!$C$78,""))))</f>
         <v/>
       </c>
       <c r="W6" s="2" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=5,Input_Bulanan!$F$74=5),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=5,Input_Bulanan!$F$75=5),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=5,Input_Bulanan!$F$76=5),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=5,Input_Bulanan!$F$77=5),Input_Bulanan!$C$77,""))))</f>
+        <f>IF(AND(Input_Bulanan!$G$75=5,Input_Bulanan!$F$75=5),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=5,Input_Bulanan!$F$76=5),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=5,Input_Bulanan!$F$77=5),Input_Bulanan!$C$77,IF(AND(Input_Bulanan!$G$78=5,Input_Bulanan!$F$78=5),Input_Bulanan!$C$78,""))))</f>
         <v>C2</v>
       </c>
     </row>
     <row r="7" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B7" s="157"/>
+      <c r="B7" s="159"/>
       <c r="C7" s="116"/>
       <c r="D7" s="116"/>
       <c r="E7" s="116"/>
-      <c r="F7" s="158"/>
-      <c r="G7" s="146"/>
-      <c r="H7" s="147"/>
-      <c r="I7" s="147"/>
-      <c r="J7" s="147"/>
-      <c r="K7" s="147"/>
-      <c r="L7" s="148"/>
-      <c r="M7" s="157"/>
+      <c r="F7" s="160"/>
+      <c r="G7" s="161"/>
+      <c r="H7" s="145"/>
+      <c r="I7" s="145"/>
+      <c r="J7" s="145"/>
+      <c r="K7" s="145"/>
+      <c r="L7" s="146"/>
+      <c r="M7" s="159"/>
       <c r="N7" s="116"/>
       <c r="O7" s="116"/>
       <c r="P7" s="116"/>
-      <c r="Q7" s="158"/>
+      <c r="Q7" s="160"/>
       <c r="R7" s="1" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
       <c r="S7" s="6" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=1,Input_Bulanan!$F$74=4),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=1,Input_Bulanan!$F$75=4),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=1,Input_Bulanan!$F$76=4),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=1,Input_Bulanan!$F$77=4),Input_Bulanan!$C$77,""))))</f>
+        <f>IF(AND(Input_Bulanan!$G$75=1,Input_Bulanan!$F$75=4),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=1,Input_Bulanan!$F$76=4),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=1,Input_Bulanan!$F$77=4),Input_Bulanan!$C$77,IF(AND(Input_Bulanan!$G$78=1,Input_Bulanan!$F$78=4),Input_Bulanan!$C$78,""))))</f>
         <v/>
       </c>
       <c r="T7" s="5" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=2,Input_Bulanan!$F$74=4),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=2,Input_Bulanan!$F$75=4),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=2,Input_Bulanan!$F$76=4),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=2,Input_Bulanan!$F$77=4),Input_Bulanan!$C$77,""))))</f>
+        <f>IF(AND(Input_Bulanan!$G$75=2,Input_Bulanan!$F$75=4),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=2,Input_Bulanan!$F$76=4),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=2,Input_Bulanan!$F$77=4),Input_Bulanan!$C$77,IF(AND(Input_Bulanan!$G$78=2,Input_Bulanan!$F$78=4),Input_Bulanan!$C$78,""))))</f>
         <v/>
       </c>
       <c r="U7" s="3" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=3,Input_Bulanan!$F$74=4),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=3,Input_Bulanan!$F$75=4),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=3,Input_Bulanan!$F$76=4),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=3,Input_Bulanan!$F$77=4),Input_Bulanan!$C$77,""))))</f>
+        <f>IF(AND(Input_Bulanan!$G$75=3,Input_Bulanan!$F$75=4),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=3,Input_Bulanan!$F$76=4),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=3,Input_Bulanan!$F$77=4),Input_Bulanan!$C$77,IF(AND(Input_Bulanan!$G$78=3,Input_Bulanan!$F$78=4),Input_Bulanan!$C$78,""))))</f>
         <v/>
       </c>
       <c r="V7" s="4" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=4,Input_Bulanan!$F$74=4),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=4,Input_Bulanan!$F$75=4),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=4,Input_Bulanan!$F$76=4),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=4,Input_Bulanan!$F$77=4),Input_Bulanan!$C$77,""))))</f>
+        <f>IF(AND(Input_Bulanan!$G$75=4,Input_Bulanan!$F$75=4),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=4,Input_Bulanan!$F$76=4),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=4,Input_Bulanan!$F$77=4),Input_Bulanan!$C$77,IF(AND(Input_Bulanan!$G$78=4,Input_Bulanan!$F$78=4),Input_Bulanan!$C$78,""))))</f>
         <v>C3</v>
       </c>
       <c r="W7" s="2" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=5,Input_Bulanan!$F$74=4),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=5,Input_Bulanan!$F$75=4),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=5,Input_Bulanan!$F$76=4),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=5,Input_Bulanan!$F$77=4),Input_Bulanan!$C$77,""))))</f>
+        <f>IF(AND(Input_Bulanan!$G$75=5,Input_Bulanan!$F$75=4),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=5,Input_Bulanan!$F$76=4),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=5,Input_Bulanan!$F$77=4),Input_Bulanan!$C$77,IF(AND(Input_Bulanan!$G$78=5,Input_Bulanan!$F$78=4),Input_Bulanan!$C$78,""))))</f>
         <v>C1</v>
       </c>
     </row>
     <row r="8" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B8" s="157"/>
+      <c r="B8" s="159"/>
       <c r="C8" s="116"/>
       <c r="D8" s="116"/>
       <c r="E8" s="116"/>
-      <c r="F8" s="158"/>
-      <c r="G8" s="175" t="s">
+      <c r="F8" s="160"/>
+      <c r="G8" s="162" t="s">
         <v>54</v>
       </c>
-      <c r="H8" s="144"/>
-      <c r="I8" s="144"/>
-      <c r="J8" s="144"/>
-      <c r="K8" s="150">
+      <c r="H8" s="158"/>
+      <c r="I8" s="158"/>
+      <c r="J8" s="158"/>
+      <c r="K8" s="143">
         <f>Input_Bulanan!D32</f>
         <v>0.70650000000000013</v>
       </c>
-      <c r="L8" s="145"/>
-      <c r="M8" s="157"/>
+      <c r="L8" s="144"/>
+      <c r="M8" s="159"/>
       <c r="N8" s="116"/>
       <c r="O8" s="116"/>
       <c r="P8" s="116"/>
-      <c r="Q8" s="158"/>
+      <c r="Q8" s="160"/>
       <c r="R8" s="1" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
       <c r="S8" s="6" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=1,Input_Bulanan!$F$74=3),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=1,Input_Bulanan!$F$75=3),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=1,Input_Bulanan!$F$76=3),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=1,Input_Bulanan!$F$77=3),Input_Bulanan!$C$77,""))))</f>
+        <f>IF(AND(Input_Bulanan!$G$75=1,Input_Bulanan!$F$75=3),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=1,Input_Bulanan!$F$76=3),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=1,Input_Bulanan!$F$77=3),Input_Bulanan!$C$77,IF(AND(Input_Bulanan!$G$78=1,Input_Bulanan!$F$78=3),Input_Bulanan!$C$78,""))))</f>
         <v/>
       </c>
       <c r="T8" s="5" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=2,Input_Bulanan!$F$74=3),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=2,Input_Bulanan!$F$75=3),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=2,Input_Bulanan!$F$76=3),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=2,Input_Bulanan!$F$77=3),Input_Bulanan!$C$77,""))))</f>
+        <f>IF(AND(Input_Bulanan!$G$75=2,Input_Bulanan!$F$75=3),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=2,Input_Bulanan!$F$76=3),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=2,Input_Bulanan!$F$77=3),Input_Bulanan!$C$77,IF(AND(Input_Bulanan!$G$78=2,Input_Bulanan!$F$78=3),Input_Bulanan!$C$78,""))))</f>
         <v/>
       </c>
       <c r="U8" s="3" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=3,Input_Bulanan!$F$74=3),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=3,Input_Bulanan!$F$75=3),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=3,Input_Bulanan!$F$76=3),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=3,Input_Bulanan!$F$77=3),Input_Bulanan!$C$77,""))))</f>
+        <f>IF(AND(Input_Bulanan!$G$75=3,Input_Bulanan!$F$75=3),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=3,Input_Bulanan!$F$76=3),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=3,Input_Bulanan!$F$77=3),Input_Bulanan!$C$77,IF(AND(Input_Bulanan!$G$78=3,Input_Bulanan!$F$78=3),Input_Bulanan!$C$78,""))))</f>
         <v>C4</v>
       </c>
       <c r="V8" s="4" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=4,Input_Bulanan!$F$74=3),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=4,Input_Bulanan!$F$75=3),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=4,Input_Bulanan!$F$76=3),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=4,Input_Bulanan!$F$77=3),Input_Bulanan!$C$77,""))))</f>
+        <f>IF(AND(Input_Bulanan!$G$75=4,Input_Bulanan!$F$75=3),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=4,Input_Bulanan!$F$76=3),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=4,Input_Bulanan!$F$77=3),Input_Bulanan!$C$77,IF(AND(Input_Bulanan!$G$78=4,Input_Bulanan!$F$78=3),Input_Bulanan!$C$78,""))))</f>
         <v/>
       </c>
       <c r="W8" s="2" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=5,Input_Bulanan!$F$74=3),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=5,Input_Bulanan!$F$75=3),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=5,Input_Bulanan!$F$76=3),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=5,Input_Bulanan!$F$77=3),Input_Bulanan!$C$77,""))))</f>
+        <f>IF(AND(Input_Bulanan!$G$75=5,Input_Bulanan!$F$75=3),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=5,Input_Bulanan!$F$76=3),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=5,Input_Bulanan!$F$77=3),Input_Bulanan!$C$77,IF(AND(Input_Bulanan!$G$78=5,Input_Bulanan!$F$78=3),Input_Bulanan!$C$78,""))))</f>
         <v/>
       </c>
     </row>
     <row r="9" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B9" s="146"/>
-      <c r="C9" s="147"/>
-      <c r="D9" s="147"/>
-      <c r="E9" s="147"/>
-      <c r="F9" s="148"/>
-      <c r="G9" s="146"/>
-      <c r="H9" s="147"/>
-      <c r="I9" s="147"/>
-      <c r="J9" s="147"/>
-      <c r="K9" s="147"/>
-      <c r="L9" s="148"/>
-      <c r="M9" s="146"/>
-      <c r="N9" s="147"/>
-      <c r="O9" s="147"/>
-      <c r="P9" s="147"/>
-      <c r="Q9" s="148"/>
+      <c r="B9" s="161"/>
+      <c r="C9" s="145"/>
+      <c r="D9" s="145"/>
+      <c r="E9" s="145"/>
+      <c r="F9" s="146"/>
+      <c r="G9" s="161"/>
+      <c r="H9" s="145"/>
+      <c r="I9" s="145"/>
+      <c r="J9" s="145"/>
+      <c r="K9" s="145"/>
+      <c r="L9" s="146"/>
+      <c r="M9" s="161"/>
+      <c r="N9" s="145"/>
+      <c r="O9" s="145"/>
+      <c r="P9" s="145"/>
+      <c r="Q9" s="146"/>
       <c r="R9" s="1" t="s">
-        <v>395</v>
+        <v>391</v>
       </c>
       <c r="S9" s="6" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=1,Input_Bulanan!$F$74=2),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=1,Input_Bulanan!$F$75=2),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=1,Input_Bulanan!$F$76=2),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=1,Input_Bulanan!$F$77=2),Input_Bulanan!$C$77,""))))</f>
+        <f>IF(AND(Input_Bulanan!$G$75=1,Input_Bulanan!$F$75=2),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=1,Input_Bulanan!$F$76=2),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=1,Input_Bulanan!$F$77=2),Input_Bulanan!$C$77,IF(AND(Input_Bulanan!$G$78=1,Input_Bulanan!$F$78=2),Input_Bulanan!$C$78,""))))</f>
         <v/>
       </c>
       <c r="T9" s="5" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=2,Input_Bulanan!$F$74=2),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=2,Input_Bulanan!$F$75=2),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=2,Input_Bulanan!$F$76=2),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=2,Input_Bulanan!$F$77=2),Input_Bulanan!$C$77,""))))</f>
+        <f>IF(AND(Input_Bulanan!$G$75=2,Input_Bulanan!$F$75=2),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=2,Input_Bulanan!$F$76=2),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=2,Input_Bulanan!$F$77=2),Input_Bulanan!$C$77,IF(AND(Input_Bulanan!$G$78=2,Input_Bulanan!$F$78=2),Input_Bulanan!$C$78,""))))</f>
         <v/>
       </c>
       <c r="U9" s="5" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=3,Input_Bulanan!$F$74=2),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=3,Input_Bulanan!$F$75=2),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=3,Input_Bulanan!$F$76=2),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=3,Input_Bulanan!$F$77=2),Input_Bulanan!$C$77,""))))</f>
+        <f>IF(AND(Input_Bulanan!$G$75=3,Input_Bulanan!$F$75=2),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=3,Input_Bulanan!$F$76=2),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=3,Input_Bulanan!$F$77=2),Input_Bulanan!$C$77,IF(AND(Input_Bulanan!$G$78=3,Input_Bulanan!$F$78=2),Input_Bulanan!$C$78,""))))</f>
         <v/>
       </c>
       <c r="V9" s="4" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=4,Input_Bulanan!$F$74=2),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=4,Input_Bulanan!$F$75=2),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=4,Input_Bulanan!$F$76=2),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=4,Input_Bulanan!$F$77=2),Input_Bulanan!$C$77,""))))</f>
+        <f>IF(AND(Input_Bulanan!$G$75=4,Input_Bulanan!$F$75=2),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=4,Input_Bulanan!$F$76=2),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=4,Input_Bulanan!$F$77=2),Input_Bulanan!$C$77,IF(AND(Input_Bulanan!$G$78=4,Input_Bulanan!$F$78=2),Input_Bulanan!$C$78,""))))</f>
         <v/>
       </c>
       <c r="W9" s="2" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=5,Input_Bulanan!$F$74=2),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=5,Input_Bulanan!$F$75=2),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=5,Input_Bulanan!$F$76=2),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=5,Input_Bulanan!$F$77=2),Input_Bulanan!$C$77,""))))</f>
+        <f>IF(AND(Input_Bulanan!$G$75=5,Input_Bulanan!$F$75=2),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=5,Input_Bulanan!$F$76=2),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=5,Input_Bulanan!$F$77=2),Input_Bulanan!$C$77,IF(AND(Input_Bulanan!$G$78=5,Input_Bulanan!$F$78=2),Input_Bulanan!$C$78,""))))</f>
         <v/>
       </c>
     </row>
     <row r="10" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B10" s="143" t="str">
+      <c r="B10" s="193" t="str">
         <f>IF(B6&gt;=0.9,"HIJAU - SEHAT",IF(B6&gt;=0.75,"KUNING - PANTAU",IF(B6&gt;=0.6,"ORANYE - WASPADA","MERAH - KRITIS")))</f>
         <v>ORANYE - WASPADA</v>
       </c>
-      <c r="C10" s="144"/>
-      <c r="D10" s="144"/>
-      <c r="E10" s="144"/>
-      <c r="F10" s="145"/>
-      <c r="G10" s="175" t="s">
+      <c r="C10" s="158"/>
+      <c r="D10" s="158"/>
+      <c r="E10" s="158"/>
+      <c r="F10" s="144"/>
+      <c r="G10" s="162" t="s">
         <v>55</v>
       </c>
-      <c r="H10" s="144"/>
-      <c r="I10" s="144"/>
-      <c r="J10" s="144"/>
-      <c r="K10" s="150">
-        <f>Input_Bulanan!D41</f>
-        <v>0.62</v>
-      </c>
-      <c r="L10" s="145"/>
-      <c r="M10" s="177" t="str">
-        <f>"Skor Komposit: "&amp;TEXT(Input_Bulanan!D47,"0,00")&amp;" / 100"</f>
-        <v>Skor Komposit: 49,24 / 100</v>
-      </c>
-      <c r="N10" s="144"/>
-      <c r="O10" s="144"/>
-      <c r="P10" s="144"/>
-      <c r="Q10" s="145"/>
+      <c r="H10" s="158"/>
+      <c r="I10" s="158"/>
+      <c r="J10" s="158"/>
+      <c r="K10" s="143">
+        <f>Input_Bulanan!D42</f>
+        <v>0.6</v>
+      </c>
+      <c r="L10" s="144"/>
+      <c r="M10" s="170" t="str">
+        <f>"Skor Komposit: "&amp;TEXT(Input_Bulanan!D48,"0,00")&amp;" / 100"</f>
+        <v>Skor Komposit: 48,84 / 100</v>
+      </c>
+      <c r="N10" s="158"/>
+      <c r="O10" s="158"/>
+      <c r="P10" s="158"/>
+      <c r="Q10" s="144"/>
       <c r="R10" s="1" t="s">
-        <v>396</v>
+        <v>392</v>
       </c>
       <c r="S10" s="6" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=1,Input_Bulanan!$F$74=1),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=1,Input_Bulanan!$F$75=1),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=1,Input_Bulanan!$F$76=1),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=1,Input_Bulanan!$F$77=1),Input_Bulanan!$C$77,""))))</f>
+        <f>IF(AND(Input_Bulanan!$G$75=1,Input_Bulanan!$F$75=1),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=1,Input_Bulanan!$F$76=1),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=1,Input_Bulanan!$F$77=1),Input_Bulanan!$C$77,IF(AND(Input_Bulanan!$G$78=1,Input_Bulanan!$F$78=1),Input_Bulanan!$C$78,""))))</f>
         <v/>
       </c>
       <c r="T10" s="6" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=2,Input_Bulanan!$F$74=1),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=2,Input_Bulanan!$F$75=1),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=2,Input_Bulanan!$F$76=1),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=2,Input_Bulanan!$F$77=1),Input_Bulanan!$C$77,""))))</f>
+        <f>IF(AND(Input_Bulanan!$G$75=2,Input_Bulanan!$F$75=1),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=2,Input_Bulanan!$F$76=1),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=2,Input_Bulanan!$F$77=1),Input_Bulanan!$C$77,IF(AND(Input_Bulanan!$G$78=2,Input_Bulanan!$F$78=1),Input_Bulanan!$C$78,""))))</f>
         <v/>
       </c>
       <c r="U10" s="5" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=3,Input_Bulanan!$F$74=1),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=3,Input_Bulanan!$F$75=1),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=3,Input_Bulanan!$F$76=1),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=3,Input_Bulanan!$F$77=1),Input_Bulanan!$C$77,""))))</f>
+        <f>IF(AND(Input_Bulanan!$G$75=3,Input_Bulanan!$F$75=1),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=3,Input_Bulanan!$F$76=1),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=3,Input_Bulanan!$F$77=1),Input_Bulanan!$C$77,IF(AND(Input_Bulanan!$G$78=3,Input_Bulanan!$F$78=1),Input_Bulanan!$C$78,""))))</f>
         <v/>
       </c>
       <c r="V10" s="3" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=4,Input_Bulanan!$F$74=1),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=4,Input_Bulanan!$F$75=1),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=4,Input_Bulanan!$F$76=1),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=4,Input_Bulanan!$F$77=1),Input_Bulanan!$C$77,""))))</f>
+        <f>IF(AND(Input_Bulanan!$G$75=4,Input_Bulanan!$F$75=1),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=4,Input_Bulanan!$F$76=1),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=4,Input_Bulanan!$F$77=1),Input_Bulanan!$C$77,IF(AND(Input_Bulanan!$G$78=4,Input_Bulanan!$F$78=1),Input_Bulanan!$C$78,""))))</f>
         <v/>
       </c>
       <c r="W10" s="2" t="str">
-        <f>IF(AND(Input_Bulanan!$G$74=5,Input_Bulanan!$F$74=1),Input_Bulanan!$C$74,IF(AND(Input_Bulanan!$G$75=5,Input_Bulanan!$F$75=1),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=5,Input_Bulanan!$F$76=1),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=5,Input_Bulanan!$F$77=1),Input_Bulanan!$C$77,""))))</f>
+        <f>IF(AND(Input_Bulanan!$G$75=5,Input_Bulanan!$F$75=1),Input_Bulanan!$C$75,IF(AND(Input_Bulanan!$G$76=5,Input_Bulanan!$F$76=1),Input_Bulanan!$C$76,IF(AND(Input_Bulanan!$G$77=5,Input_Bulanan!$F$77=1),Input_Bulanan!$C$77,IF(AND(Input_Bulanan!$G$78=5,Input_Bulanan!$F$78=1),Input_Bulanan!$C$78,""))))</f>
         <v/>
       </c>
     </row>
     <row r="11" spans="2:23" ht="12" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B11" s="146"/>
-      <c r="C11" s="147"/>
-      <c r="D11" s="147"/>
-      <c r="E11" s="147"/>
-      <c r="F11" s="148"/>
-      <c r="G11" s="146"/>
-      <c r="H11" s="147"/>
-      <c r="I11" s="147"/>
-      <c r="J11" s="147"/>
-      <c r="K11" s="147"/>
-      <c r="L11" s="148"/>
-      <c r="M11" s="146"/>
-      <c r="N11" s="147"/>
-      <c r="O11" s="147"/>
-      <c r="P11" s="147"/>
-      <c r="Q11" s="148"/>
+      <c r="B11" s="161"/>
+      <c r="C11" s="145"/>
+      <c r="D11" s="145"/>
+      <c r="E11" s="145"/>
+      <c r="F11" s="146"/>
+      <c r="G11" s="161"/>
+      <c r="H11" s="145"/>
+      <c r="I11" s="145"/>
+      <c r="J11" s="145"/>
+      <c r="K11" s="145"/>
+      <c r="L11" s="146"/>
+      <c r="M11" s="161"/>
+      <c r="N11" s="145"/>
+      <c r="O11" s="145"/>
+      <c r="P11" s="145"/>
+      <c r="Q11" s="146"/>
       <c r="R11" s="7" t="s">
-        <v>397</v>
+        <v>393</v>
       </c>
       <c r="S11" s="8">
         <v>1</v>
@@ -3804,14 +3814,14 @@
       </c>
     </row>
     <row r="12" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B12" s="154" t="s">
+      <c r="B12" s="164" t="s">
         <v>56</v>
       </c>
       <c r="C12" s="118"/>
       <c r="D12" s="118"/>
       <c r="E12" s="118"/>
       <c r="F12" s="120"/>
-      <c r="G12" s="154" t="s">
+      <c r="G12" s="164" t="s">
         <v>57</v>
       </c>
       <c r="H12" s="118"/>
@@ -3819,14 +3829,14 @@
       <c r="J12" s="118"/>
       <c r="K12" s="118"/>
       <c r="L12" s="120"/>
-      <c r="M12" s="154" t="s">
+      <c r="M12" s="164" t="s">
         <v>58</v>
       </c>
       <c r="N12" s="118"/>
       <c r="O12" s="118"/>
       <c r="P12" s="118"/>
       <c r="Q12" s="120"/>
-      <c r="R12" s="154" t="s">
+      <c r="R12" s="164" t="s">
         <v>59</v>
       </c>
       <c r="S12" s="118"/>
@@ -3836,43 +3846,43 @@
       <c r="W12" s="120"/>
     </row>
     <row r="13" spans="2:23" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B13" s="153" t="s">
+      <c r="B13" s="150" t="s">
         <v>60</v>
       </c>
       <c r="C13" s="118"/>
       <c r="D13" s="120"/>
-      <c r="E13" s="173">
+      <c r="E13" s="167">
         <f>Input_Bulanan!D12</f>
         <v>1</v>
       </c>
       <c r="F13" s="120"/>
-      <c r="G13" s="141" t="s">
+      <c r="G13" s="189" t="s">
         <v>61</v>
       </c>
       <c r="H13" s="118"/>
       <c r="I13" s="120"/>
-      <c r="J13" s="164">
+      <c r="J13" s="169">
         <f>Input_Bulanan!D8</f>
         <v>100</v>
       </c>
       <c r="K13" s="118"/>
       <c r="L13" s="120"/>
-      <c r="M13" s="159" t="s">
+      <c r="M13" s="163" t="s">
         <v>62</v>
       </c>
       <c r="N13" s="118"/>
       <c r="O13" s="120"/>
-      <c r="P13" s="163">
-        <f>Input_Bulanan!D51</f>
+      <c r="P13" s="190">
+        <f>Input_Bulanan!D52</f>
         <v>5</v>
       </c>
       <c r="Q13" s="120"/>
       <c r="R13" s="9" t="str">
-        <f>Input_Bulanan!C74</f>
+        <f>Input_Bulanan!C75</f>
         <v>C1</v>
       </c>
-      <c r="S13" s="162" t="str">
-        <f>Input_Bulanan!D74&amp;"  |  L="&amp;Input_Bulanan!F74&amp;", C="&amp;Input_Bulanan!G74&amp;", Skala="&amp;Input_Bulanan!H74&amp;" -&gt; "&amp;Input_Bulanan!I74</f>
+      <c r="S13" s="174" t="str">
+        <f>Input_Bulanan!D75&amp;"  |  L="&amp;Input_Bulanan!F75&amp;", C="&amp;Input_Bulanan!G75&amp;", Skala="&amp;Input_Bulanan!H75&amp;" -&gt; "&amp;Input_Bulanan!I75</f>
         <v>Salt Supply Disruption (gangguan pasokan garam industri)  |  L=4, C=5, Skala=24 -&gt; High</v>
       </c>
       <c r="T13" s="118"/>
@@ -3881,43 +3891,43 @@
       <c r="W13" s="118"/>
     </row>
     <row r="14" spans="2:23" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B14" s="153" t="s">
+      <c r="B14" s="150" t="s">
         <v>63</v>
       </c>
       <c r="C14" s="118"/>
       <c r="D14" s="120"/>
-      <c r="E14" s="173">
+      <c r="E14" s="167">
         <f>Input_Bulanan!D14</f>
         <v>1</v>
       </c>
       <c r="F14" s="120"/>
-      <c r="G14" s="141" t="s">
+      <c r="G14" s="189" t="s">
         <v>64</v>
       </c>
       <c r="H14" s="118"/>
       <c r="I14" s="120"/>
-      <c r="J14" s="164">
+      <c r="J14" s="169">
         <f>Input_Bulanan!D9</f>
         <v>100</v>
       </c>
       <c r="K14" s="118"/>
       <c r="L14" s="120"/>
-      <c r="M14" s="159" t="s">
+      <c r="M14" s="163" t="s">
         <v>65</v>
       </c>
       <c r="N14" s="118"/>
       <c r="O14" s="120"/>
-      <c r="P14" s="178">
-        <f>Input_Bulanan!D52</f>
+      <c r="P14" s="172">
+        <f>Input_Bulanan!D53</f>
         <v>11</v>
       </c>
       <c r="Q14" s="120"/>
       <c r="R14" s="9" t="str">
-        <f>Input_Bulanan!C75</f>
+        <f>Input_Bulanan!C76</f>
         <v>C2</v>
       </c>
-      <c r="S14" s="162" t="str">
-        <f>Input_Bulanan!D75&amp;"  |  L="&amp;Input_Bulanan!F75&amp;", C="&amp;Input_Bulanan!G75&amp;", Skala="&amp;Input_Bulanan!H75&amp;" -&gt; "&amp;Input_Bulanan!I75</f>
+      <c r="S14" s="174" t="str">
+        <f>Input_Bulanan!D76&amp;"  |  L="&amp;Input_Bulanan!F76&amp;", C="&amp;Input_Bulanan!G76&amp;", Skala="&amp;Input_Bulanan!H76&amp;" -&gt; "&amp;Input_Bulanan!I76</f>
         <v>Commissioning Delay (keterlambatan commissioning)  |  L=5, C=5, Skala=25 -&gt; High</v>
       </c>
       <c r="T14" s="118"/>
@@ -3926,43 +3936,43 @@
       <c r="W14" s="118"/>
     </row>
     <row r="15" spans="2:23" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B15" s="153" t="s">
+      <c r="B15" s="150" t="s">
         <v>66</v>
       </c>
       <c r="C15" s="118"/>
       <c r="D15" s="120"/>
-      <c r="E15" s="176">
+      <c r="E15" s="152">
         <f>Input_Bulanan!D13</f>
         <v>0</v>
       </c>
       <c r="F15" s="120"/>
-      <c r="G15" s="141" t="s">
+      <c r="G15" s="189" t="s">
         <v>67</v>
       </c>
       <c r="H15" s="118"/>
       <c r="I15" s="120"/>
-      <c r="J15" s="164">
+      <c r="J15" s="169">
         <f>Input_Bulanan!D10</f>
         <v>100</v>
       </c>
       <c r="K15" s="118"/>
       <c r="L15" s="120"/>
-      <c r="M15" s="159" t="s">
+      <c r="M15" s="163" t="s">
         <v>68</v>
       </c>
       <c r="N15" s="118"/>
       <c r="O15" s="120"/>
-      <c r="P15" s="165">
-        <f>Input_Bulanan!D53</f>
+      <c r="P15" s="191">
+        <f>Input_Bulanan!D54</f>
         <v>18</v>
       </c>
       <c r="Q15" s="120"/>
       <c r="R15" s="9" t="str">
-        <f>Input_Bulanan!C76</f>
+        <f>Input_Bulanan!C77</f>
         <v>C3</v>
       </c>
-      <c r="S15" s="162" t="str">
-        <f>Input_Bulanan!D76&amp;"  |  L="&amp;Input_Bulanan!F76&amp;", C="&amp;Input_Bulanan!G76&amp;", Skala="&amp;Input_Bulanan!H76&amp;" -&gt; "&amp;Input_Bulanan!I76</f>
+      <c r="S15" s="174" t="str">
+        <f>Input_Bulanan!D77&amp;"  |  L="&amp;Input_Bulanan!F77&amp;", C="&amp;Input_Bulanan!G77&amp;", Skala="&amp;Input_Bulanan!H77&amp;" -&gt; "&amp;Input_Bulanan!I77</f>
         <v>EPC Interface Issue (isu EPC interface lintas kontraktor)  |  L=4, C=4, Skala=19 -&gt; Moderate to High</v>
       </c>
       <c r="T15" s="118"/>
@@ -3971,17 +3981,17 @@
       <c r="W15" s="118"/>
     </row>
     <row r="16" spans="2:23" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B16" s="153" t="s">
+      <c r="B16" s="150" t="s">
         <v>69</v>
       </c>
       <c r="C16" s="118"/>
       <c r="D16" s="120"/>
-      <c r="E16" s="176">
+      <c r="E16" s="152">
         <f>Input_Bulanan!D15</f>
         <v>0</v>
       </c>
       <c r="F16" s="120"/>
-      <c r="G16" s="194" t="s">
+      <c r="G16" s="153" t="s">
         <v>70</v>
       </c>
       <c r="H16" s="118"/>
@@ -3989,22 +3999,22 @@
       <c r="J16" s="118"/>
       <c r="K16" s="118"/>
       <c r="L16" s="120"/>
-      <c r="M16" s="159" t="s">
+      <c r="M16" s="163" t="s">
         <v>71</v>
       </c>
       <c r="N16" s="118"/>
       <c r="O16" s="120"/>
-      <c r="P16" s="193">
-        <f>Input_Bulanan!D54</f>
+      <c r="P16" s="147">
+        <f>Input_Bulanan!D55</f>
         <v>4</v>
       </c>
       <c r="Q16" s="120"/>
       <c r="R16" s="9" t="str">
-        <f>Input_Bulanan!C77</f>
+        <f>Input_Bulanan!C78</f>
         <v>C4</v>
       </c>
-      <c r="S16" s="162" t="str">
-        <f>Input_Bulanan!D77&amp;"  |  L="&amp;Input_Bulanan!F77&amp;", C="&amp;Input_Bulanan!G77&amp;", Skala="&amp;Input_Bulanan!H77&amp;" -&gt; "&amp;Input_Bulanan!I77</f>
+      <c r="S16" s="174" t="str">
+        <f>Input_Bulanan!D78&amp;"  |  L="&amp;Input_Bulanan!F78&amp;", C="&amp;Input_Bulanan!G78&amp;", Skala="&amp;Input_Bulanan!H78&amp;" -&gt; "&amp;Input_Bulanan!I78</f>
         <v>Long Lead Equipment (keterlambatan peralatan utama)  |  L=3, C=3, Skala=13 -&gt; Moderate</v>
       </c>
       <c r="T16" s="118"/>
@@ -4014,13 +4024,13 @@
     </row>
     <row r="17" spans="2:23" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="L17" s="106"/>
-      <c r="M17" s="159" t="s">
+      <c r="M17" s="163" t="s">
         <v>72</v>
       </c>
       <c r="N17" s="118"/>
       <c r="O17" s="120"/>
-      <c r="P17" s="193">
-        <f>Input_Bulanan!D55</f>
+      <c r="P17" s="147">
+        <f>Input_Bulanan!D56</f>
         <v>3</v>
       </c>
       <c r="Q17" s="120"/>
@@ -4031,8 +4041,8 @@
       </c>
       <c r="N18" s="103"/>
       <c r="O18" s="104"/>
-      <c r="P18" s="192">
-        <f>Input_Bulanan!D56</f>
+      <c r="P18" s="151">
+        <f>Input_Bulanan!D57</f>
         <v>41</v>
       </c>
       <c r="Q18" s="120"/>
@@ -4056,20 +4066,20 @@
       <c r="Q19" s="116"/>
     </row>
     <row r="20" spans="2:23" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B20" s="179" t="s">
+      <c r="B20" s="175" t="s">
         <v>74</v>
       </c>
-      <c r="C20" s="180"/>
-      <c r="D20" s="180"/>
-      <c r="E20" s="180"/>
-      <c r="F20" s="180"/>
-      <c r="G20" s="180"/>
-      <c r="H20" s="180"/>
-      <c r="I20" s="180"/>
-      <c r="J20" s="180"/>
-      <c r="K20" s="180"/>
-      <c r="L20" s="181"/>
-      <c r="M20" s="174" t="s">
+      <c r="C20" s="176"/>
+      <c r="D20" s="176"/>
+      <c r="E20" s="176"/>
+      <c r="F20" s="176"/>
+      <c r="G20" s="176"/>
+      <c r="H20" s="176"/>
+      <c r="I20" s="176"/>
+      <c r="J20" s="176"/>
+      <c r="K20" s="176"/>
+      <c r="L20" s="177"/>
+      <c r="M20" s="188" t="s">
         <v>75</v>
       </c>
       <c r="N20" s="118"/>
@@ -4078,93 +4088,93 @@
       <c r="Q20" s="120"/>
     </row>
     <row r="21" spans="2:23" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B21" s="182"/>
-      <c r="C21" s="183"/>
-      <c r="D21" s="183"/>
-      <c r="E21" s="183"/>
-      <c r="F21" s="183"/>
-      <c r="G21" s="183"/>
-      <c r="H21" s="183"/>
-      <c r="I21" s="183"/>
-      <c r="J21" s="183"/>
-      <c r="K21" s="183"/>
-      <c r="L21" s="184"/>
-      <c r="M21" s="153" t="s">
+      <c r="B21" s="178"/>
+      <c r="C21" s="179"/>
+      <c r="D21" s="179"/>
+      <c r="E21" s="179"/>
+      <c r="F21" s="179"/>
+      <c r="G21" s="179"/>
+      <c r="H21" s="179"/>
+      <c r="I21" s="179"/>
+      <c r="J21" s="179"/>
+      <c r="K21" s="179"/>
+      <c r="L21" s="180"/>
+      <c r="M21" s="150" t="s">
         <v>76</v>
       </c>
       <c r="N21" s="118"/>
       <c r="O21" s="120"/>
-      <c r="P21" s="151">
-        <f>Input_Bulanan!D59</f>
+      <c r="P21" s="165">
+        <f>Input_Bulanan!D60</f>
         <v>0.82</v>
       </c>
       <c r="Q21" s="120"/>
     </row>
     <row r="22" spans="2:23" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B22" s="182"/>
-      <c r="C22" s="183"/>
-      <c r="D22" s="183"/>
-      <c r="E22" s="183"/>
-      <c r="F22" s="183"/>
-      <c r="G22" s="183"/>
-      <c r="H22" s="183"/>
-      <c r="I22" s="183"/>
-      <c r="J22" s="183"/>
-      <c r="K22" s="183"/>
-      <c r="L22" s="184"/>
-      <c r="M22" s="153" t="s">
+      <c r="B22" s="178"/>
+      <c r="C22" s="179"/>
+      <c r="D22" s="179"/>
+      <c r="E22" s="179"/>
+      <c r="F22" s="179"/>
+      <c r="G22" s="179"/>
+      <c r="H22" s="179"/>
+      <c r="I22" s="179"/>
+      <c r="J22" s="179"/>
+      <c r="K22" s="179"/>
+      <c r="L22" s="180"/>
+      <c r="M22" s="150" t="s">
         <v>77</v>
       </c>
       <c r="N22" s="118"/>
       <c r="O22" s="120"/>
-      <c r="P22" s="151">
-        <f>Input_Bulanan!D60</f>
+      <c r="P22" s="165">
+        <f>Input_Bulanan!D61</f>
         <v>0.18</v>
       </c>
       <c r="Q22" s="120"/>
     </row>
     <row r="23" spans="2:23" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B23" s="182"/>
-      <c r="C23" s="183"/>
-      <c r="D23" s="183"/>
-      <c r="E23" s="183"/>
-      <c r="F23" s="183"/>
-      <c r="G23" s="183"/>
-      <c r="H23" s="183"/>
-      <c r="I23" s="183"/>
-      <c r="J23" s="183"/>
-      <c r="K23" s="183"/>
-      <c r="L23" s="184"/>
-      <c r="M23" s="153" t="s">
+      <c r="B23" s="178"/>
+      <c r="C23" s="179"/>
+      <c r="D23" s="179"/>
+      <c r="E23" s="179"/>
+      <c r="F23" s="179"/>
+      <c r="G23" s="179"/>
+      <c r="H23" s="179"/>
+      <c r="I23" s="179"/>
+      <c r="J23" s="179"/>
+      <c r="K23" s="179"/>
+      <c r="L23" s="180"/>
+      <c r="M23" s="150" t="s">
         <v>78</v>
       </c>
       <c r="N23" s="118"/>
       <c r="O23" s="120"/>
-      <c r="P23" s="151">
-        <f>Input_Bulanan!D61</f>
+      <c r="P23" s="165">
+        <f>Input_Bulanan!D62</f>
         <v>0.76</v>
       </c>
       <c r="Q23" s="120"/>
     </row>
     <row r="24" spans="2:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B24" s="185"/>
-      <c r="C24" s="186"/>
-      <c r="D24" s="186"/>
-      <c r="E24" s="186"/>
-      <c r="F24" s="186"/>
-      <c r="G24" s="186"/>
-      <c r="H24" s="186"/>
-      <c r="I24" s="186"/>
-      <c r="J24" s="186"/>
-      <c r="K24" s="186"/>
-      <c r="L24" s="187"/>
-      <c r="M24" s="153" t="s">
+      <c r="B24" s="181"/>
+      <c r="C24" s="182"/>
+      <c r="D24" s="182"/>
+      <c r="E24" s="182"/>
+      <c r="F24" s="182"/>
+      <c r="G24" s="182"/>
+      <c r="H24" s="182"/>
+      <c r="I24" s="182"/>
+      <c r="J24" s="182"/>
+      <c r="K24" s="182"/>
+      <c r="L24" s="183"/>
+      <c r="M24" s="150" t="s">
         <v>79</v>
       </c>
       <c r="N24" s="118"/>
       <c r="O24" s="120"/>
-      <c r="P24" s="170">
-        <f>Input_Bulanan!D62</f>
+      <c r="P24" s="185">
+        <f>Input_Bulanan!D63</f>
         <v>5</v>
       </c>
       <c r="Q24" s="120"/>
@@ -4194,7 +4204,7 @@
       <c r="W25" s="116"/>
     </row>
     <row r="26" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B26" s="160" t="s">
+      <c r="B26" s="168" t="s">
         <v>80</v>
       </c>
       <c r="C26" s="118"/>
@@ -4220,20 +4230,20 @@
       <c r="W26" s="120"/>
     </row>
     <row r="27" spans="2:23" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B27" s="149" t="s">
+      <c r="B27" s="166" t="s">
         <v>81</v>
       </c>
       <c r="C27" s="118"/>
       <c r="D27" s="118"/>
       <c r="E27" s="118"/>
       <c r="F27" s="120"/>
-      <c r="G27" s="149" t="s">
+      <c r="G27" s="166" t="s">
         <v>82</v>
       </c>
       <c r="H27" s="118"/>
       <c r="I27" s="118"/>
       <c r="J27" s="120"/>
-      <c r="K27" s="149" t="s">
+      <c r="K27" s="166" t="s">
         <v>83</v>
       </c>
       <c r="L27" s="120"/>
@@ -4246,7 +4256,7 @@
       <c r="O27" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="P27" s="149" t="s">
+      <c r="P27" s="166" t="s">
         <v>87</v>
       </c>
       <c r="Q27" s="118"/>
@@ -4258,37 +4268,37 @@
       <c r="W27" s="120"/>
     </row>
     <row r="28" spans="2:23" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B28" s="141" t="s">
+      <c r="B28" s="189" t="s">
         <v>88</v>
       </c>
       <c r="C28" s="118"/>
       <c r="D28" s="118"/>
       <c r="E28" s="118"/>
       <c r="F28" s="120"/>
-      <c r="G28" s="152" t="s">
+      <c r="G28" s="142" t="s">
         <v>89</v>
       </c>
       <c r="H28" s="118"/>
       <c r="I28" s="118"/>
       <c r="J28" s="120"/>
-      <c r="K28" s="171">
-        <f>Input_Bulanan!E66</f>
+      <c r="K28" s="186">
+        <f>Input_Bulanan!E67</f>
         <v>46113</v>
       </c>
       <c r="L28" s="120"/>
       <c r="M28" s="107" t="str">
-        <f>IF(Input_Bulanan!H66="Aman","V","")</f>
+        <f>IF(Input_Bulanan!H67="Aman","V","")</f>
         <v>V</v>
       </c>
       <c r="N28" s="107" t="str">
-        <f>IF(Input_Bulanan!H66="Waspada","V","")</f>
+        <f>IF(Input_Bulanan!H67="Waspada","V","")</f>
         <v/>
       </c>
       <c r="O28" s="107" t="str">
-        <f>IF(Input_Bulanan!H66="Bahaya","V","")</f>
+        <f>IF(Input_Bulanan!H67="Bahaya","V","")</f>
         <v/>
       </c>
-      <c r="P28" s="191" t="s">
+      <c r="P28" s="141" t="s">
         <v>90</v>
       </c>
       <c r="Q28" s="118"/>
@@ -4300,37 +4310,37 @@
       <c r="W28" s="120"/>
     </row>
     <row r="29" spans="2:23" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B29" s="155" t="s">
+      <c r="B29" s="140" t="s">
         <v>91</v>
       </c>
       <c r="C29" s="118"/>
       <c r="D29" s="118"/>
       <c r="E29" s="118"/>
       <c r="F29" s="120"/>
-      <c r="G29" s="167" t="s">
+      <c r="G29" s="173" t="s">
         <v>92</v>
       </c>
       <c r="H29" s="118"/>
       <c r="I29" s="118"/>
       <c r="J29" s="120"/>
-      <c r="K29" s="142">
-        <f>Input_Bulanan!E67</f>
+      <c r="K29" s="148">
+        <f>Input_Bulanan!E68</f>
         <v>0.88</v>
       </c>
       <c r="L29" s="120"/>
       <c r="M29" s="107" t="str">
-        <f>IF(Input_Bulanan!H67="Aman","V","")</f>
+        <f>IF(Input_Bulanan!H68="Aman","V","")</f>
         <v/>
       </c>
       <c r="N29" s="107" t="str">
-        <f>IF(Input_Bulanan!H67="Waspada","V","")</f>
+        <f>IF(Input_Bulanan!H68="Waspada","V","")</f>
         <v/>
       </c>
       <c r="O29" s="107" t="str">
-        <f>IF(Input_Bulanan!H67="Bahaya","V","")</f>
+        <f>IF(Input_Bulanan!H68="Bahaya","V","")</f>
         <v>V</v>
       </c>
-      <c r="P29" s="166" t="s">
+      <c r="P29" s="171" t="s">
         <v>93</v>
       </c>
       <c r="Q29" s="118"/>
@@ -4342,37 +4352,37 @@
       <c r="W29" s="120"/>
     </row>
     <row r="30" spans="2:23" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B30" s="141" t="s">
+      <c r="B30" s="189" t="s">
         <v>94</v>
       </c>
       <c r="C30" s="118"/>
       <c r="D30" s="118"/>
       <c r="E30" s="118"/>
       <c r="F30" s="120"/>
-      <c r="G30" s="152" t="s">
+      <c r="G30" s="142" t="s">
         <v>95</v>
       </c>
       <c r="H30" s="118"/>
       <c r="I30" s="118"/>
       <c r="J30" s="120"/>
-      <c r="K30" s="172">
-        <f>Input_Bulanan!E68</f>
+      <c r="K30" s="187">
+        <f>Input_Bulanan!E69</f>
         <v>0.6</v>
       </c>
       <c r="L30" s="120"/>
       <c r="M30" s="107" t="str">
-        <f>IF(Input_Bulanan!H68="Aman","V","")</f>
+        <f>IF(Input_Bulanan!H69="Aman","V","")</f>
         <v/>
       </c>
       <c r="N30" s="107" t="str">
-        <f>IF(Input_Bulanan!H68="Waspada","V","")</f>
+        <f>IF(Input_Bulanan!H69="Waspada","V","")</f>
         <v/>
       </c>
       <c r="O30" s="107" t="str">
-        <f>IF(Input_Bulanan!H68="Bahaya","V","")</f>
+        <f>IF(Input_Bulanan!H69="Bahaya","V","")</f>
         <v>V</v>
       </c>
-      <c r="P30" s="191" t="s">
+      <c r="P30" s="141" t="s">
         <v>96</v>
       </c>
       <c r="Q30" s="118"/>
@@ -4384,20 +4394,20 @@
       <c r="W30" s="120"/>
     </row>
     <row r="31" spans="2:23" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B31" s="155" t="s">
+      <c r="B31" s="140" t="s">
         <v>97</v>
       </c>
       <c r="C31" s="118"/>
       <c r="D31" s="118"/>
       <c r="E31" s="118"/>
       <c r="F31" s="120"/>
-      <c r="G31" s="167" t="s">
+      <c r="G31" s="173" t="s">
         <v>98</v>
       </c>
       <c r="H31" s="118"/>
       <c r="I31" s="118"/>
       <c r="J31" s="120"/>
-      <c r="K31" s="142" t="e">
+      <c r="K31" s="148" t="e">
         <f>Input_Bulanan!#REF!</f>
         <v>#REF!</v>
       </c>
@@ -4414,7 +4424,7 @@
         <f>IF(Input_Bulanan!#REF!="Bahaya","V","")</f>
         <v>#REF!</v>
       </c>
-      <c r="P31" s="166" t="s">
+      <c r="P31" s="171" t="s">
         <v>99</v>
       </c>
       <c r="Q31" s="118"/>
@@ -4426,20 +4436,20 @@
       <c r="W31" s="120"/>
     </row>
     <row r="32" spans="2:23" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B32" s="141" t="s">
+      <c r="B32" s="189" t="s">
         <v>100</v>
       </c>
       <c r="C32" s="118"/>
       <c r="D32" s="118"/>
       <c r="E32" s="118"/>
       <c r="F32" s="120"/>
-      <c r="G32" s="152" t="s">
+      <c r="G32" s="142" t="s">
         <v>101</v>
       </c>
       <c r="H32" s="118"/>
       <c r="I32" s="118"/>
       <c r="J32" s="120"/>
-      <c r="K32" s="168" t="e">
+      <c r="K32" s="192" t="e">
         <f>Input_Bulanan!#REF!</f>
         <v>#REF!</v>
       </c>
@@ -4456,7 +4466,7 @@
         <f>IF(Input_Bulanan!#REF!="Bahaya","V","")</f>
         <v>#REF!</v>
       </c>
-      <c r="P32" s="191" t="s">
+      <c r="P32" s="141" t="s">
         <v>102</v>
       </c>
       <c r="Q32" s="118"/>
@@ -4468,20 +4478,20 @@
       <c r="W32" s="120"/>
     </row>
     <row r="33" spans="2:23" x14ac:dyDescent="0.45">
-      <c r="B33" s="155" t="s">
+      <c r="B33" s="140" t="s">
         <v>103</v>
       </c>
       <c r="C33" s="118"/>
       <c r="D33" s="118"/>
       <c r="E33" s="118"/>
       <c r="F33" s="120"/>
-      <c r="G33" s="167" t="s">
+      <c r="G33" s="173" t="s">
         <v>104</v>
       </c>
       <c r="H33" s="118"/>
       <c r="I33" s="118"/>
       <c r="J33" s="120"/>
-      <c r="K33" s="142" t="e">
+      <c r="K33" s="148" t="e">
         <f>Input_Bulanan!#REF!</f>
         <v>#REF!</v>
       </c>
@@ -4498,7 +4508,7 @@
         <f>IF(Input_Bulanan!#REF!="Bahaya","V","")</f>
         <v>#REF!</v>
       </c>
-      <c r="P33" s="166" t="s">
+      <c r="P33" s="171" t="s">
         <v>105</v>
       </c>
       <c r="Q33" s="118"/>
@@ -4534,7 +4544,7 @@
       <c r="W34" s="116"/>
     </row>
     <row r="35" spans="2:23" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B35" s="160" t="s">
+      <c r="B35" s="168" t="s">
         <v>106</v>
       </c>
       <c r="C35" s="118"/>
@@ -4560,7 +4570,7 @@
       <c r="W35" s="120"/>
     </row>
     <row r="36" spans="2:23" ht="33" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B36" s="161" t="str">
+      <c r="B36" s="156" t="str">
         <f>"Prioritas 1—2: [1] " &amp; INDEX(Risk_Action_Tracker!E$6:E$15, MATCH(LARGE(Risk_Action_Tracker!Z$6:Z$15, 1), Risk_Action_Tracker!Z$6:Z$15, 0)) &amp; " · [2] " &amp; INDEX(Risk_Action_Tracker!E$6:E$15, MATCH(LARGE(Risk_Action_Tracker!Z$6:Z$15, 2), Risk_Action_Tracker!Z$6:Z$15, 0))</f>
         <v>Prioritas 1—2: [1] Mengesahkan pembentukan tim Interface Coordinator dan menerapkan Interface Management Plan (IMP) yang mengikat seluruh kontraktor; mengharuskan Rekind menyelaraskan jadwal penyusunan gambar detail dengan kemajuan ISBL EPC-A. · [2] Memberikan dispensasi perpanjangan jaminan pelaksanaan secara terkendali; meminta Parent Company Guarantee dari PT Perusahaan Induk X (Persero) untuk menjamin ketersediaan pendanaan bila Rekind menghadapi kendala likuiditas.</v>
       </c>
@@ -4587,7 +4597,7 @@
       <c r="W36" s="120"/>
     </row>
     <row r="37" spans="2:23" ht="42.4" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B37" s="161" t="s">
+      <c r="B37" s="156" t="s">
         <v>107</v>
       </c>
       <c r="C37" s="118"/>
@@ -4614,24 +4624,70 @@
     </row>
   </sheetData>
   <mergeCells count="98">
-    <mergeCell ref="B33:F33"/>
-    <mergeCell ref="P30:W30"/>
-    <mergeCell ref="G30:J30"/>
-    <mergeCell ref="M19:Q19"/>
-    <mergeCell ref="K6:L7"/>
-    <mergeCell ref="P16:Q16"/>
-    <mergeCell ref="P32:W32"/>
-    <mergeCell ref="K31:L31"/>
-    <mergeCell ref="B29:F29"/>
-    <mergeCell ref="R5:W5"/>
-    <mergeCell ref="P28:W28"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="G28:J28"/>
-    <mergeCell ref="P18:Q18"/>
-    <mergeCell ref="P17:Q17"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="B19:L19"/>
-    <mergeCell ref="G16:L16"/>
+    <mergeCell ref="M4:W4"/>
+    <mergeCell ref="G13:I13"/>
+    <mergeCell ref="K33:L33"/>
+    <mergeCell ref="B10:F11"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="K8:L9"/>
+    <mergeCell ref="G15:I15"/>
+    <mergeCell ref="P22:Q22"/>
+    <mergeCell ref="G32:J32"/>
+    <mergeCell ref="M21:O21"/>
+    <mergeCell ref="G5:L5"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="K29:L29"/>
+    <mergeCell ref="B6:F9"/>
+    <mergeCell ref="M17:O17"/>
+    <mergeCell ref="B26:W26"/>
+    <mergeCell ref="B36:W36"/>
+    <mergeCell ref="S14:W14"/>
+    <mergeCell ref="K10:L11"/>
+    <mergeCell ref="M24:O24"/>
+    <mergeCell ref="S13:W13"/>
+    <mergeCell ref="M12:Q12"/>
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="S15:W15"/>
+    <mergeCell ref="P13:Q13"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="J13:L13"/>
+    <mergeCell ref="P15:Q15"/>
+    <mergeCell ref="P31:W31"/>
+    <mergeCell ref="G31:J31"/>
+    <mergeCell ref="K32:L32"/>
+    <mergeCell ref="B1:W1"/>
+    <mergeCell ref="P24:Q24"/>
+    <mergeCell ref="K28:L28"/>
+    <mergeCell ref="J15:L15"/>
+    <mergeCell ref="K30:L30"/>
+    <mergeCell ref="M22:O22"/>
+    <mergeCell ref="P29:W29"/>
+    <mergeCell ref="G29:J29"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="R12:W12"/>
+    <mergeCell ref="M5:Q5"/>
+    <mergeCell ref="M15:O15"/>
+    <mergeCell ref="M20:Q20"/>
+    <mergeCell ref="G14:I14"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B35:W35"/>
+    <mergeCell ref="G6:J7"/>
+    <mergeCell ref="B25:W25"/>
+    <mergeCell ref="M14:O14"/>
+    <mergeCell ref="M23:O23"/>
+    <mergeCell ref="K27:L27"/>
+    <mergeCell ref="G12:L12"/>
+    <mergeCell ref="J14:L14"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="M10:Q11"/>
+    <mergeCell ref="P33:W33"/>
+    <mergeCell ref="P14:Q14"/>
+    <mergeCell ref="G33:J33"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="S16:W16"/>
+    <mergeCell ref="B20:L24"/>
     <mergeCell ref="B2:W2"/>
     <mergeCell ref="B34:W34"/>
     <mergeCell ref="B4:L4"/>
@@ -4648,70 +4704,24 @@
     <mergeCell ref="G27:J27"/>
     <mergeCell ref="P23:Q23"/>
     <mergeCell ref="E13:F13"/>
-    <mergeCell ref="B35:W35"/>
-    <mergeCell ref="G6:J7"/>
-    <mergeCell ref="B25:W25"/>
-    <mergeCell ref="M14:O14"/>
-    <mergeCell ref="M23:O23"/>
-    <mergeCell ref="K27:L27"/>
-    <mergeCell ref="G12:L12"/>
-    <mergeCell ref="J14:L14"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="M10:Q11"/>
-    <mergeCell ref="P33:W33"/>
-    <mergeCell ref="P14:Q14"/>
-    <mergeCell ref="G33:J33"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="S16:W16"/>
-    <mergeCell ref="B20:L24"/>
-    <mergeCell ref="B1:W1"/>
-    <mergeCell ref="P24:Q24"/>
-    <mergeCell ref="K28:L28"/>
-    <mergeCell ref="J15:L15"/>
-    <mergeCell ref="K30:L30"/>
-    <mergeCell ref="M22:O22"/>
-    <mergeCell ref="P29:W29"/>
-    <mergeCell ref="G29:J29"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="R12:W12"/>
-    <mergeCell ref="M5:Q5"/>
-    <mergeCell ref="M15:O15"/>
-    <mergeCell ref="M20:Q20"/>
-    <mergeCell ref="G14:I14"/>
-    <mergeCell ref="B5:F5"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="B36:W36"/>
-    <mergeCell ref="S14:W14"/>
-    <mergeCell ref="K10:L11"/>
-    <mergeCell ref="M24:O24"/>
-    <mergeCell ref="S13:W13"/>
-    <mergeCell ref="M12:Q12"/>
-    <mergeCell ref="B32:F32"/>
-    <mergeCell ref="B28:F28"/>
-    <mergeCell ref="S15:W15"/>
-    <mergeCell ref="P13:Q13"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="J13:L13"/>
-    <mergeCell ref="P15:Q15"/>
-    <mergeCell ref="P31:W31"/>
-    <mergeCell ref="G31:J31"/>
-    <mergeCell ref="K32:L32"/>
-    <mergeCell ref="M4:W4"/>
-    <mergeCell ref="G13:I13"/>
-    <mergeCell ref="K33:L33"/>
-    <mergeCell ref="B10:F11"/>
-    <mergeCell ref="B27:F27"/>
-    <mergeCell ref="K8:L9"/>
-    <mergeCell ref="G15:I15"/>
-    <mergeCell ref="P22:Q22"/>
-    <mergeCell ref="G32:J32"/>
-    <mergeCell ref="M21:O21"/>
-    <mergeCell ref="G5:L5"/>
-    <mergeCell ref="B31:F31"/>
-    <mergeCell ref="K29:L29"/>
-    <mergeCell ref="B6:F9"/>
-    <mergeCell ref="M17:O17"/>
-    <mergeCell ref="B26:W26"/>
+    <mergeCell ref="R5:W5"/>
+    <mergeCell ref="P28:W28"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="G28:J28"/>
+    <mergeCell ref="P18:Q18"/>
+    <mergeCell ref="P17:Q17"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="B19:L19"/>
+    <mergeCell ref="G16:L16"/>
+    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="P30:W30"/>
+    <mergeCell ref="G30:J30"/>
+    <mergeCell ref="M19:Q19"/>
+    <mergeCell ref="K6:L7"/>
+    <mergeCell ref="P16:Q16"/>
+    <mergeCell ref="P32:W32"/>
+    <mergeCell ref="K31:L31"/>
+    <mergeCell ref="B29:F29"/>
   </mergeCells>
   <conditionalFormatting sqref="B10:F11">
     <cfRule type="expression" dxfId="11" priority="2">
@@ -4790,8 +4800,8 @@
       <c r="E2" s="13"/>
     </row>
     <row r="3" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="135" t="s">
-        <v>374</v>
+      <c r="A3" s="127" t="s">
+        <v>370</v>
       </c>
       <c r="B3" s="116"/>
       <c r="C3" s="116"/>
@@ -4799,7 +4809,7 @@
       <c r="E3" s="116"/>
     </row>
     <row r="5" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="119" t="s">
+      <c r="A5" s="122" t="s">
         <v>109</v>
       </c>
       <c r="B5" s="118"/>
@@ -4872,7 +4882,7 @@
         <v>0.2</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="45.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -4889,7 +4899,7 @@
         <v>0.2</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="45.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -4906,7 +4916,7 @@
         <v>0.2</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.45">
@@ -4918,7 +4928,7 @@
       </c>
     </row>
     <row r="14" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A14" s="139" t="s">
+      <c r="A14" s="115" t="s">
         <v>130</v>
       </c>
       <c r="B14" s="116"/>
@@ -4927,7 +4937,7 @@
       <c r="E14" s="116"/>
     </row>
     <row r="15" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="115" t="s">
+      <c r="A15" s="136" t="s">
         <v>131</v>
       </c>
       <c r="B15" s="116"/>
@@ -4936,7 +4946,7 @@
       <c r="E15" s="116"/>
     </row>
     <row r="17" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="119" t="s">
+      <c r="A17" s="122" t="s">
         <v>132</v>
       </c>
       <c r="B17" s="118"/>
@@ -4951,7 +4961,7 @@
       <c r="B18" s="14" t="s">
         <v>133</v>
       </c>
-      <c r="C18" s="137" t="s">
+      <c r="C18" s="124" t="s">
         <v>134</v>
       </c>
       <c r="D18" s="118"/>
@@ -4964,7 +4974,7 @@
       <c r="B19" s="110">
         <v>0.25</v>
       </c>
-      <c r="C19" s="124" t="s">
+      <c r="C19" s="125" t="s">
         <v>136</v>
       </c>
       <c r="D19" s="118"/>
@@ -4990,7 +5000,7 @@
       <c r="B21" s="110">
         <v>0.2</v>
       </c>
-      <c r="C21" s="124" t="s">
+      <c r="C21" s="125" t="s">
         <v>140</v>
       </c>
       <c r="D21" s="118"/>
@@ -5016,14 +5026,14 @@
       <c r="B23" s="110">
         <v>0.15</v>
       </c>
-      <c r="C23" s="124" t="s">
+      <c r="C23" s="125" t="s">
         <v>144</v>
       </c>
       <c r="D23" s="118"/>
       <c r="E23" s="118"/>
     </row>
     <row r="25" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A25" s="119" t="s">
+      <c r="A25" s="122" t="s">
         <v>145</v>
       </c>
       <c r="B25" s="118"/>
@@ -5038,7 +5048,7 @@
       <c r="B26" s="14" t="s">
         <v>133</v>
       </c>
-      <c r="C26" s="137" t="s">
+      <c r="C26" s="124" t="s">
         <v>134</v>
       </c>
       <c r="D26" s="118"/>
@@ -5051,7 +5061,7 @@
       <c r="B27" s="110">
         <v>0.25</v>
       </c>
-      <c r="C27" s="124" t="s">
+      <c r="C27" s="125" t="s">
         <v>147</v>
       </c>
       <c r="D27" s="118"/>
@@ -5077,7 +5087,7 @@
       <c r="B29" s="110">
         <v>0.35</v>
       </c>
-      <c r="C29" s="124" t="s">
+      <c r="C29" s="125" t="s">
         <v>151</v>
       </c>
       <c r="D29" s="118"/>
@@ -5097,7 +5107,7 @@
       <c r="E30" s="118"/>
     </row>
     <row r="32" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A32" s="119" t="s">
+      <c r="A32" s="122" t="s">
         <v>154</v>
       </c>
       <c r="B32" s="118"/>
@@ -5112,7 +5122,7 @@
       <c r="B33" s="14" t="s">
         <v>133</v>
       </c>
-      <c r="C33" s="137" t="s">
+      <c r="C33" s="124" t="s">
         <v>134</v>
       </c>
       <c r="D33" s="118"/>
@@ -5138,7 +5148,7 @@
       <c r="B35" s="110">
         <v>0.2</v>
       </c>
-      <c r="C35" s="124" t="s">
+      <c r="C35" s="125" t="s">
         <v>158</v>
       </c>
       <c r="D35" s="118"/>
@@ -5164,7 +5174,7 @@
       <c r="B37" s="110">
         <v>0.2</v>
       </c>
-      <c r="C37" s="124" t="s">
+      <c r="C37" s="125" t="s">
         <v>162</v>
       </c>
       <c r="D37" s="118"/>
@@ -5184,7 +5194,7 @@
       <c r="E38" s="118"/>
     </row>
     <row r="40" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A40" s="119" t="s">
+      <c r="A40" s="122" t="s">
         <v>165</v>
       </c>
       <c r="B40" s="118"/>
@@ -5333,7 +5343,7 @@
       </c>
     </row>
     <row r="49" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A49" s="119" t="s">
+      <c r="A49" s="122" t="s">
         <v>202</v>
       </c>
       <c r="B49" s="118"/>
@@ -5342,8 +5352,8 @@
       <c r="E49" s="120"/>
     </row>
     <row r="50" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A50" s="136" t="s">
-        <v>375</v>
+      <c r="A50" s="131" t="s">
+        <v>371</v>
       </c>
       <c r="B50" s="116"/>
       <c r="C50" s="116"/>
@@ -5357,7 +5367,7 @@
       <c r="B51" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="C51" s="123" t="s">
+      <c r="C51" s="119" t="s">
         <v>204</v>
       </c>
       <c r="D51" s="118"/>
@@ -5370,7 +5380,7 @@
       <c r="B52" s="30" t="s">
         <v>205</v>
       </c>
-      <c r="C52" s="122" t="s">
+      <c r="C52" s="123" t="s">
         <v>206</v>
       </c>
       <c r="D52" s="118"/>
@@ -5383,7 +5393,7 @@
       <c r="B53" s="32" t="s">
         <v>207</v>
       </c>
-      <c r="C53" s="129" t="s">
+      <c r="C53" s="121" t="s">
         <v>208</v>
       </c>
       <c r="D53" s="118"/>
@@ -5396,7 +5406,7 @@
       <c r="B54" s="30" t="s">
         <v>209</v>
       </c>
-      <c r="C54" s="122" t="s">
+      <c r="C54" s="123" t="s">
         <v>210</v>
       </c>
       <c r="D54" s="118"/>
@@ -5409,7 +5419,7 @@
       <c r="B55" s="32" t="s">
         <v>211</v>
       </c>
-      <c r="C55" s="129" t="s">
+      <c r="C55" s="121" t="s">
         <v>212</v>
       </c>
       <c r="D55" s="118"/>
@@ -5422,14 +5432,14 @@
       <c r="B56" s="30" t="s">
         <v>213</v>
       </c>
-      <c r="C56" s="122" t="s">
+      <c r="C56" s="123" t="s">
         <v>214</v>
       </c>
       <c r="D56" s="118"/>
       <c r="E56" s="118"/>
     </row>
     <row r="58" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A58" s="119" t="s">
+      <c r="A58" s="122" t="s">
         <v>215</v>
       </c>
       <c r="B58" s="118"/>
@@ -5444,7 +5454,7 @@
       <c r="B59" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="C59" s="123" t="s">
+      <c r="C59" s="119" t="s">
         <v>217</v>
       </c>
       <c r="D59" s="118"/>
@@ -5457,7 +5467,7 @@
       <c r="B60" s="30" t="s">
         <v>218</v>
       </c>
-      <c r="C60" s="122" t="s">
+      <c r="C60" s="123" t="s">
         <v>219</v>
       </c>
       <c r="D60" s="118"/>
@@ -5470,7 +5480,7 @@
       <c r="B61" s="32" t="s">
         <v>220</v>
       </c>
-      <c r="C61" s="129" t="s">
+      <c r="C61" s="121" t="s">
         <v>221</v>
       </c>
       <c r="D61" s="118"/>
@@ -5483,7 +5493,7 @@
       <c r="B62" s="30" t="s">
         <v>222</v>
       </c>
-      <c r="C62" s="122" t="s">
+      <c r="C62" s="123" t="s">
         <v>223</v>
       </c>
       <c r="D62" s="118"/>
@@ -5496,7 +5506,7 @@
       <c r="B63" s="32" t="s">
         <v>224</v>
       </c>
-      <c r="C63" s="129" t="s">
+      <c r="C63" s="121" t="s">
         <v>225</v>
       </c>
       <c r="D63" s="118"/>
@@ -5509,15 +5519,15 @@
       <c r="B64" s="30" t="s">
         <v>226</v>
       </c>
-      <c r="C64" s="122" t="s">
+      <c r="C64" s="123" t="s">
         <v>227</v>
       </c>
       <c r="D64" s="118"/>
       <c r="E64" s="118"/>
     </row>
     <row r="66" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A66" s="119" t="s">
-        <v>376</v>
+      <c r="A66" s="122" t="s">
+        <v>372</v>
       </c>
       <c r="B66" s="118"/>
       <c r="C66" s="118"/>
@@ -5525,7 +5535,7 @@
       <c r="E66" s="120"/>
     </row>
     <row r="67" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A67" s="138" t="s">
+      <c r="A67" s="132" t="s">
         <v>228</v>
       </c>
       <c r="B67" s="116"/>
@@ -5540,7 +5550,7 @@
       <c r="B68" s="9" t="s">
         <v>230</v>
       </c>
-      <c r="C68" s="123" t="s">
+      <c r="C68" s="119" t="s">
         <v>231</v>
       </c>
       <c r="D68" s="118"/>
@@ -5553,7 +5563,7 @@
       <c r="B69" s="37" t="s">
         <v>232</v>
       </c>
-      <c r="C69" s="127" t="s">
+      <c r="C69" s="126" t="s">
         <v>233</v>
       </c>
       <c r="D69" s="118"/>
@@ -5566,7 +5576,7 @@
       <c r="B70" s="37" t="s">
         <v>234</v>
       </c>
-      <c r="C70" s="127" t="s">
+      <c r="C70" s="126" t="s">
         <v>235</v>
       </c>
       <c r="D70" s="118"/>
@@ -5579,7 +5589,7 @@
       <c r="B71" s="37" t="s">
         <v>236</v>
       </c>
-      <c r="C71" s="127" t="s">
+      <c r="C71" s="126" t="s">
         <v>237</v>
       </c>
       <c r="D71" s="118"/>
@@ -5592,7 +5602,7 @@
       <c r="B72" s="37" t="s">
         <v>238</v>
       </c>
-      <c r="C72" s="127" t="s">
+      <c r="C72" s="126" t="s">
         <v>239</v>
       </c>
       <c r="D72" s="118"/>
@@ -5605,14 +5615,14 @@
       <c r="B73" s="37" t="s">
         <v>240</v>
       </c>
-      <c r="C73" s="127" t="s">
+      <c r="C73" s="126" t="s">
         <v>241</v>
       </c>
       <c r="D73" s="118"/>
       <c r="E73" s="118"/>
     </row>
     <row r="75" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A75" s="119" t="s">
+      <c r="A75" s="122" t="s">
         <v>242</v>
       </c>
       <c r="B75" s="118"/>
@@ -5627,7 +5637,7 @@
       <c r="B76" s="111">
         <v>0.4</v>
       </c>
-      <c r="C76" s="122" t="s">
+      <c r="C76" s="123" t="s">
         <v>244</v>
       </c>
       <c r="D76" s="118"/>
@@ -5640,7 +5650,7 @@
       <c r="B77" s="110">
         <v>0.4</v>
       </c>
-      <c r="C77" s="129" t="s">
+      <c r="C77" s="121" t="s">
         <v>246</v>
       </c>
       <c r="D77" s="118"/>
@@ -5653,14 +5663,14 @@
       <c r="B78" s="111">
         <v>0.2</v>
       </c>
-      <c r="C78" s="122" t="s">
-        <v>372</v>
+      <c r="C78" s="123" t="s">
+        <v>368</v>
       </c>
       <c r="D78" s="118"/>
       <c r="E78" s="118"/>
     </row>
     <row r="79" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A79" s="125" t="s">
+      <c r="A79" s="138" t="s">
         <v>248</v>
       </c>
       <c r="B79" s="116"/>
@@ -5670,7 +5680,7 @@
     </row>
     <row r="81" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A81" s="42" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
     </row>
     <row r="82" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.45"/>
@@ -5687,8 +5697,8 @@
       <c r="F86" s="44"/>
     </row>
     <row r="87" spans="1:6" ht="43.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A87" s="128" t="s">
-        <v>378</v>
+      <c r="A87" s="133" t="s">
+        <v>374</v>
       </c>
       <c r="B87" s="116"/>
       <c r="C87" s="116"/>
@@ -6217,8 +6227,8 @@
       </c>
     </row>
     <row r="116" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A116" s="128" t="s">
-        <v>379</v>
+      <c r="A116" s="133" t="s">
+        <v>375</v>
       </c>
       <c r="B116" s="116"/>
       <c r="C116" s="116"/>
@@ -6237,7 +6247,7 @@
       <c r="F118" s="44"/>
     </row>
     <row r="119" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A119" s="128" t="s">
+      <c r="A119" s="133" t="s">
         <v>261</v>
       </c>
       <c r="B119" s="116"/>
@@ -6250,7 +6260,7 @@
       <c r="A121" s="51" t="s">
         <v>262</v>
       </c>
-      <c r="B121" s="131" t="s">
+      <c r="B121" s="135" t="s">
         <v>263</v>
       </c>
       <c r="C121" s="116"/>
@@ -6263,33 +6273,33 @@
       <c r="A122" s="52" t="s">
         <v>84</v>
       </c>
-      <c r="B122" s="132" t="s">
+      <c r="B122" s="128" t="s">
         <v>265</v>
       </c>
-      <c r="C122" s="133"/>
-      <c r="D122" s="134"/>
+      <c r="C122" s="129"/>
+      <c r="D122" s="130"/>
       <c r="E122" s="53"/>
     </row>
     <row r="123" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A123" s="54" t="s">
         <v>85</v>
       </c>
-      <c r="B123" s="132" t="s">
+      <c r="B123" s="128" t="s">
         <v>266</v>
       </c>
-      <c r="C123" s="133"/>
-      <c r="D123" s="134"/>
+      <c r="C123" s="129"/>
+      <c r="D123" s="130"/>
       <c r="E123" s="53"/>
     </row>
     <row r="124" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A124" s="55" t="s">
         <v>86</v>
       </c>
-      <c r="B124" s="132" t="s">
+      <c r="B124" s="128" t="s">
         <v>267</v>
       </c>
-      <c r="C124" s="133"/>
-      <c r="D124" s="134"/>
+      <c r="C124" s="129"/>
+      <c r="D124" s="130"/>
       <c r="E124" s="53"/>
     </row>
     <row r="127" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -6303,7 +6313,7 @@
       <c r="F127" s="94"/>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A129" s="126" t="s">
+      <c r="A129" s="139" t="s">
         <v>269</v>
       </c>
       <c r="B129" s="116"/>
@@ -6377,7 +6387,7 @@
         <v>247</v>
       </c>
       <c r="B133" s="96" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="C133" s="96" t="s">
         <v>285</v>
@@ -6393,7 +6403,7 @@
       </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A136" s="121" t="s">
+      <c r="A136" s="137" t="s">
         <v>288</v>
       </c>
       <c r="B136" s="116"/>
@@ -6404,7 +6414,7 @@
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A139" s="93" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
       <c r="B139" s="94"/>
       <c r="C139" s="94"/>
@@ -6413,8 +6423,8 @@
       <c r="F139" s="94"/>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A141" s="130" t="s">
-        <v>381</v>
+      <c r="A141" s="134" t="s">
+        <v>377</v>
       </c>
       <c r="B141" s="116"/>
       <c r="C141" s="116"/>
@@ -6490,6 +6500,53 @@
     </row>
   </sheetData>
   <mergeCells count="63">
+    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="A49:E49"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A136:F136"/>
+    <mergeCell ref="C56:E56"/>
+    <mergeCell ref="C59:E59"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="A79:E79"/>
+    <mergeCell ref="C51:E51"/>
+    <mergeCell ref="A129:F129"/>
+    <mergeCell ref="C60:E60"/>
+    <mergeCell ref="C36:E36"/>
+    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="C76:E76"/>
+    <mergeCell ref="C71:E71"/>
+    <mergeCell ref="C52:E52"/>
+    <mergeCell ref="A116:F116"/>
+    <mergeCell ref="C61:E61"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="A141:F141"/>
+    <mergeCell ref="C70:E70"/>
+    <mergeCell ref="A75:E75"/>
+    <mergeCell ref="A66:E66"/>
+    <mergeCell ref="B121:D121"/>
+    <mergeCell ref="B122:D122"/>
+    <mergeCell ref="A119:F119"/>
+    <mergeCell ref="A58:E58"/>
+    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="A87:F87"/>
+    <mergeCell ref="C63:E63"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="C38:E38"/>
+    <mergeCell ref="B124:D124"/>
+    <mergeCell ref="C72:E72"/>
+    <mergeCell ref="A50:E50"/>
+    <mergeCell ref="C28:E28"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="C37:E37"/>
+    <mergeCell ref="C53:E53"/>
+    <mergeCell ref="B123:D123"/>
+    <mergeCell ref="C69:E69"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="C78:E78"/>
+    <mergeCell ref="A32:E32"/>
+    <mergeCell ref="A67:E67"/>
     <mergeCell ref="A14:E14"/>
     <mergeCell ref="C30:E30"/>
     <mergeCell ref="C68:E68"/>
@@ -6506,53 +6563,6 @@
     <mergeCell ref="A40:E40"/>
     <mergeCell ref="C73:E73"/>
     <mergeCell ref="C64:E64"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="C38:E38"/>
-    <mergeCell ref="B124:D124"/>
-    <mergeCell ref="C72:E72"/>
-    <mergeCell ref="A50:E50"/>
-    <mergeCell ref="C28:E28"/>
-    <mergeCell ref="C19:E19"/>
-    <mergeCell ref="C37:E37"/>
-    <mergeCell ref="C53:E53"/>
-    <mergeCell ref="B123:D123"/>
-    <mergeCell ref="C69:E69"/>
-    <mergeCell ref="C18:E18"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="C78:E78"/>
-    <mergeCell ref="A32:E32"/>
-    <mergeCell ref="A67:E67"/>
-    <mergeCell ref="C52:E52"/>
-    <mergeCell ref="A116:F116"/>
-    <mergeCell ref="C61:E61"/>
-    <mergeCell ref="C23:E23"/>
-    <mergeCell ref="A141:F141"/>
-    <mergeCell ref="C70:E70"/>
-    <mergeCell ref="A75:E75"/>
-    <mergeCell ref="A66:E66"/>
-    <mergeCell ref="B121:D121"/>
-    <mergeCell ref="B122:D122"/>
-    <mergeCell ref="A119:F119"/>
-    <mergeCell ref="A58:E58"/>
-    <mergeCell ref="C35:E35"/>
-    <mergeCell ref="A87:F87"/>
-    <mergeCell ref="C63:E63"/>
-    <mergeCell ref="A15:E15"/>
-    <mergeCell ref="C22:E22"/>
-    <mergeCell ref="A49:E49"/>
-    <mergeCell ref="A25:E25"/>
-    <mergeCell ref="A136:F136"/>
-    <mergeCell ref="C56:E56"/>
-    <mergeCell ref="C59:E59"/>
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="A79:E79"/>
-    <mergeCell ref="C51:E51"/>
-    <mergeCell ref="A129:F129"/>
-    <mergeCell ref="C60:E60"/>
-    <mergeCell ref="C36:E36"/>
-    <mergeCell ref="C27:E27"/>
-    <mergeCell ref="C76:E76"/>
-    <mergeCell ref="C71:E71"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -6567,7 +6577,7 @@
   <sheetPr>
     <tabColor rgb="FFF2C230"/>
   </sheetPr>
-  <dimension ref="C2:I77"/>
+  <dimension ref="C2:I78"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
@@ -6587,7 +6597,7 @@
       </c>
     </row>
     <row r="3" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C3" s="135" t="s">
+      <c r="C3" s="127" t="s">
         <v>302</v>
       </c>
       <c r="D3" s="116"/>
@@ -6597,16 +6607,16 @@
     </row>
     <row r="4" spans="3:7" x14ac:dyDescent="0.45">
       <c r="C4" s="113" t="s">
-        <v>398</v>
+        <v>394</v>
       </c>
       <c r="D4" s="114" t="s">
-        <v>399</v>
+        <v>395</v>
       </c>
       <c r="F4" s="113" t="s">
-        <v>400</v>
+        <v>396</v>
       </c>
       <c r="G4" s="114" t="s">
-        <v>401</v>
+        <v>397</v>
       </c>
     </row>
     <row r="5" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -6640,7 +6650,7 @@
         <v>100</v>
       </c>
       <c r="E8" t="s">
-        <v>366</v>
+        <v>362</v>
       </c>
     </row>
     <row r="9" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -6661,7 +6671,7 @@
     </row>
     <row r="11" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C11" s="58" t="s">
-        <v>402</v>
+        <v>398</v>
       </c>
       <c r="D11" s="59">
         <v>77.599999999999994</v>
@@ -6714,7 +6724,7 @@
     </row>
     <row r="18" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C18" s="58" t="s">
-        <v>403</v>
+        <v>399</v>
       </c>
       <c r="D18" s="62">
         <v>0.1</v>
@@ -6722,18 +6732,18 @@
     </row>
     <row r="19" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C19" s="58" t="s">
-        <v>404</v>
+        <v>400</v>
       </c>
       <c r="D19" s="62">
         <v>0.05</v>
       </c>
       <c r="E19" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
     </row>
     <row r="20" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C20" s="58" t="s">
-        <v>405</v>
+        <v>401</v>
       </c>
       <c r="D20" s="62">
         <v>0.04</v>
@@ -6741,7 +6751,7 @@
     </row>
     <row r="21" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C21" s="58" t="s">
-        <v>406</v>
+        <v>402</v>
       </c>
       <c r="D21" s="62">
         <v>0.06</v>
@@ -6757,7 +6767,7 @@
     </row>
     <row r="23" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C23" s="58" t="s">
-        <v>407</v>
+        <v>403</v>
       </c>
       <c r="D23" s="62">
         <v>0.8</v>
@@ -6783,7 +6793,7 @@
     </row>
     <row r="27" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C27" s="58" t="s">
-        <v>408</v>
+        <v>404</v>
       </c>
       <c r="D27" s="62">
         <v>0.88</v>
@@ -6794,7 +6804,7 @@
     </row>
     <row r="28" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C28" s="58" t="s">
-        <v>409</v>
+        <v>405</v>
       </c>
       <c r="D28" s="62">
         <v>0.73</v>
@@ -6805,7 +6815,7 @@
     </row>
     <row r="29" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C29" s="58" t="s">
-        <v>410</v>
+        <v>406</v>
       </c>
       <c r="D29" s="62">
         <v>0.82</v>
@@ -6822,7 +6832,7 @@
         <v>0.42</v>
       </c>
       <c r="E30" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
       <c r="F30" t="s">
         <v>311</v>
@@ -6830,7 +6840,7 @@
     </row>
     <row r="31" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C31" s="58" t="s">
-        <v>411</v>
+        <v>407</v>
       </c>
       <c r="D31" s="62">
         <v>0.4</v>
@@ -6875,7 +6885,7 @@
     </row>
     <row r="36" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C36" s="58" t="s">
-        <v>323</v>
+        <v>414</v>
       </c>
       <c r="D36" s="62">
         <v>0.6</v>
@@ -6883,7 +6893,7 @@
     </row>
     <row r="37" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C37" s="58" t="s">
-        <v>324</v>
+        <v>415</v>
       </c>
       <c r="D37" s="62">
         <v>0.6</v>
@@ -6891,7 +6901,7 @@
     </row>
     <row r="38" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C38" s="58" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="D38" s="62">
         <v>0.8</v>
@@ -6899,7 +6909,7 @@
     </row>
     <row r="39" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C39" s="58" t="s">
-        <v>326</v>
+        <v>416</v>
       </c>
       <c r="D39" s="62">
         <v>0.8</v>
@@ -6907,398 +6917,381 @@
     </row>
     <row r="40" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C40" s="58" t="s">
-        <v>327</v>
+        <v>417</v>
       </c>
       <c r="D40" s="62">
         <v>0.4</v>
       </c>
       <c r="E40" t="s">
-        <v>364</v>
+        <v>360</v>
       </c>
       <c r="F40" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
     </row>
     <row r="41" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C41" s="56" t="s">
-        <v>328</v>
-      </c>
-      <c r="D41" s="63">
-        <f>(D36*0.2+D37*0.2+D38*0.15+D39*0.2+D40*0.25)</f>
-        <v>0.62</v>
-      </c>
-    </row>
-    <row r="43" spans="3:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C43" s="195" t="s">
-        <v>329</v>
-      </c>
-      <c r="D43" s="116"/>
-      <c r="E43" s="116"/>
-      <c r="F43" s="116"/>
-      <c r="G43" s="116"/>
-    </row>
-    <row r="44" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C44" s="58" t="s">
-        <v>330</v>
-      </c>
-      <c r="D44" s="108">
+      <c r="C41" s="58" t="s">
+        <v>418</v>
+      </c>
+      <c r="D41" s="62">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="42" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C42" s="56" t="s">
+        <v>324</v>
+      </c>
+      <c r="D42" s="63">
+        <f>D36*0.15 + D37*0.15 + D38*0.15 + D39*0.15 + D40*0.2 + D41*0.2</f>
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="44" spans="3:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C44" s="195" t="s">
+        <v>325</v>
+      </c>
+      <c r="D44" s="116"/>
+      <c r="E44" s="116"/>
+      <c r="F44" s="116"/>
+      <c r="G44" s="116"/>
+    </row>
+    <row r="45" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C45" s="58" t="s">
+        <v>326</v>
+      </c>
+      <c r="D45" s="108">
         <f>D24*100</f>
         <v>21.450000000000003</v>
       </c>
     </row>
-    <row r="45" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C45" s="58" t="s">
-        <v>331</v>
-      </c>
-      <c r="D45" s="108">
+    <row r="46" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C46" s="58" t="s">
+        <v>327</v>
+      </c>
+      <c r="D46" s="108">
         <f>D32*100</f>
         <v>70.650000000000006</v>
       </c>
     </row>
-    <row r="46" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C46" s="58" t="s">
-        <v>332</v>
-      </c>
-      <c r="D46" s="108">
-        <f>D41*100</f>
-        <v>62</v>
-      </c>
-    </row>
     <row r="47" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C47" s="56" t="s">
-        <v>333</v>
-      </c>
-      <c r="D47" s="109">
-        <f>(D44*0.4)+(D45*0.4)+(D46*0.2)</f>
-        <v>49.24</v>
+      <c r="C47" s="58" t="s">
+        <v>328</v>
+      </c>
+      <c r="D47" s="108">
+        <f>D42*100</f>
+        <v>60</v>
       </c>
     </row>
     <row r="48" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C48" s="56" t="s">
-        <v>334</v>
-      </c>
-      <c r="D48" s="65" t="str">
-        <f>IF(D47&lt;=20,"Low",IF(D47&lt;=44,"Low to Moderate",IF(D47&lt;=60,"Moderate",IF(D47&lt;=76,"Moderate to High","High"))))</f>
+        <v>329</v>
+      </c>
+      <c r="D48" s="109">
+        <f>(D45*0.4)+(D46*0.4)+(D47*0.2)</f>
+        <v>48.84</v>
+      </c>
+    </row>
+    <row r="49" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C49" s="56" t="s">
+        <v>330</v>
+      </c>
+      <c r="D49" s="65" t="str">
+        <f>IF(D48&lt;=20,"Low",IF(D48&lt;=44,"Low to Moderate",IF(D48&lt;=60,"Moderate",IF(D48&lt;=76,"Moderate to High","High"))))</f>
         <v>Moderate</v>
       </c>
     </row>
-    <row r="50" spans="3:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C50" s="195" t="s">
-        <v>382</v>
-      </c>
-      <c r="D50" s="116"/>
-      <c r="E50" s="116"/>
-      <c r="F50" s="116"/>
-      <c r="G50" s="116"/>
-    </row>
-    <row r="51" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C51" s="87" t="s">
+    <row r="51" spans="3:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C51" s="195" t="s">
+        <v>378</v>
+      </c>
+      <c r="D51" s="116"/>
+      <c r="E51" s="116"/>
+      <c r="F51" s="116"/>
+      <c r="G51" s="116"/>
+    </row>
+    <row r="52" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C52" s="87" t="s">
         <v>62</v>
       </c>
-      <c r="D51" s="66">
+      <c r="D52" s="66">
         <v>5</v>
       </c>
     </row>
-    <row r="52" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C52" s="88" t="s">
+    <row r="53" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C53" s="88" t="s">
         <v>65</v>
       </c>
-      <c r="D52" s="66">
+      <c r="D53" s="66">
         <v>11</v>
       </c>
     </row>
-    <row r="53" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C53" s="89" t="s">
+    <row r="54" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C54" s="89" t="s">
         <v>68</v>
       </c>
-      <c r="D53" s="66">
+      <c r="D54" s="66">
         <v>18</v>
       </c>
     </row>
-    <row r="54" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C54" s="90" t="s">
+    <row r="55" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C55" s="90" t="s">
         <v>71</v>
       </c>
-      <c r="D54" s="66">
+      <c r="D55" s="66">
         <v>4</v>
       </c>
     </row>
-    <row r="55" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C55" s="86" t="s">
+    <row r="56" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C56" s="86" t="s">
         <v>72</v>
       </c>
-      <c r="D55" s="66">
+      <c r="D56" s="66">
         <v>3</v>
       </c>
     </row>
-    <row r="56" spans="3:7" x14ac:dyDescent="0.45">
-      <c r="C56" s="91" t="s">
+    <row r="57" spans="3:7" x14ac:dyDescent="0.45">
+      <c r="C57" s="91" t="s">
         <v>73</v>
       </c>
-      <c r="D56" s="92">
-        <f>SUM(D51:D55)</f>
+      <c r="D57" s="92">
+        <f>SUM(D52:D56)</f>
         <v>41</v>
       </c>
     </row>
-    <row r="57" spans="3:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C57" s="116"/>
-      <c r="D57" s="116"/>
-      <c r="E57" s="116"/>
-      <c r="F57" s="116"/>
-      <c r="G57" s="116"/>
-    </row>
-    <row r="58" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C58" s="195" t="s">
-        <v>335</v>
-      </c>
+    <row r="58" spans="3:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C58" s="116"/>
       <c r="D58" s="116"/>
       <c r="E58" s="116"/>
       <c r="F58" s="116"/>
       <c r="G58" s="116"/>
     </row>
     <row r="59" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C59" s="58" t="s">
-        <v>336</v>
-      </c>
-      <c r="D59" s="62">
-        <v>0.82</v>
-      </c>
-      <c r="E59" s="58" t="s">
-        <v>32</v>
-      </c>
-      <c r="F59" s="66">
-        <v>2</v>
-      </c>
+      <c r="C59" s="195" t="s">
+        <v>331</v>
+      </c>
+      <c r="D59" s="116"/>
+      <c r="E59" s="116"/>
+      <c r="F59" s="116"/>
+      <c r="G59" s="116"/>
     </row>
     <row r="60" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C60" s="58" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="D60" s="62">
-        <v>0.18</v>
+        <v>0.82</v>
       </c>
       <c r="E60" s="58" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F60" s="66">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="61" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C61" s="58" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="D61" s="62">
+        <v>0.18</v>
+      </c>
+      <c r="E61" s="58" t="s">
+        <v>34</v>
+      </c>
+      <c r="F61" s="66">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="62" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C62" s="58" t="s">
+        <v>334</v>
+      </c>
+      <c r="D62" s="62">
         <v>0.76</v>
       </c>
-      <c r="E61" s="58" t="s">
+      <c r="E62" s="58" t="s">
         <v>36</v>
       </c>
-      <c r="F61" s="66">
+      <c r="F62" s="66">
         <v>5</v>
       </c>
     </row>
-    <row r="62" spans="3:7" x14ac:dyDescent="0.45">
-      <c r="C62" s="58" t="s">
+    <row r="63" spans="3:7" x14ac:dyDescent="0.45">
+      <c r="C63" s="58" t="s">
         <v>79</v>
       </c>
-      <c r="D62" s="66">
+      <c r="D63" s="66">
         <v>5</v>
       </c>
-      <c r="E62" s="58" t="s">
+      <c r="E63" s="58" t="s">
         <v>38</v>
       </c>
-      <c r="F62" s="66">
+      <c r="F63" s="66">
         <v>4</v>
       </c>
     </row>
-    <row r="63" spans="3:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C63" s="116"/>
-      <c r="D63" s="116"/>
-      <c r="E63" s="116"/>
-      <c r="F63" s="116"/>
-      <c r="G63" s="116"/>
-    </row>
-    <row r="64" spans="3:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C64" s="195" t="s">
-        <v>339</v>
-      </c>
+    <row r="64" spans="3:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C64" s="116"/>
       <c r="D64" s="116"/>
       <c r="E64" s="116"/>
       <c r="F64" s="116"/>
       <c r="G64" s="116"/>
     </row>
     <row r="65" spans="3:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C65" s="14" t="s">
+      <c r="C65" s="195" t="s">
+        <v>335</v>
+      </c>
+      <c r="D65" s="116"/>
+      <c r="E65" s="116"/>
+      <c r="F65" s="116"/>
+      <c r="G65" s="116"/>
+    </row>
+    <row r="66" spans="3:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C66" s="14" t="s">
+        <v>336</v>
+      </c>
+      <c r="D66" s="14" t="s">
+        <v>337</v>
+      </c>
+      <c r="E66" s="14" t="s">
+        <v>338</v>
+      </c>
+      <c r="F66" s="67" t="s">
+        <v>339</v>
+      </c>
+      <c r="G66" s="67" t="s">
         <v>340</v>
       </c>
-      <c r="D65" s="14" t="s">
+      <c r="H66" s="67" t="s">
         <v>341</v>
-      </c>
-      <c r="E65" s="14" t="s">
-        <v>342</v>
-      </c>
-      <c r="F65" s="67" t="s">
-        <v>343</v>
-      </c>
-      <c r="G65" s="67" t="s">
-        <v>344</v>
-      </c>
-      <c r="H65" s="67" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="66" spans="3:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C66" s="58" t="s">
-        <v>412</v>
-      </c>
-      <c r="D66" s="68" t="s">
-        <v>413</v>
-      </c>
-      <c r="E66" s="66">
-        <v>46113</v>
-      </c>
-      <c r="F66" s="69">
-        <v>46096</v>
-      </c>
-      <c r="G66" s="69" t="s">
-        <v>414</v>
-      </c>
-      <c r="H66" s="70" t="str">
-        <f t="shared" ref="H66:H68" si="0">IF(E66&gt;=F66,"Aman",IF(E66&gt;=G66,"Waspada","Bahaya"))</f>
-        <v>Aman</v>
       </c>
     </row>
     <row r="67" spans="3:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C67" s="58" t="s">
-        <v>415</v>
+        <v>408</v>
       </c>
       <c r="D67" s="68" t="s">
-        <v>346</v>
-      </c>
-      <c r="E67" s="62">
-        <v>0.88</v>
-      </c>
-      <c r="F67" s="71">
-        <v>0.9</v>
-      </c>
-      <c r="G67" s="71" t="s">
-        <v>416</v>
+        <v>409</v>
+      </c>
+      <c r="E67" s="200">
+        <v>46113</v>
+      </c>
+      <c r="F67" s="201">
+        <v>46096</v>
+      </c>
+      <c r="G67" s="69" t="s">
+        <v>410</v>
       </c>
       <c r="H67" s="70" t="str">
-        <f t="shared" si="0"/>
-        <v>Bahaya</v>
+        <f t="shared" ref="H67:H69" si="0">IF(E67&gt;=F67,"Aman",IF(E67&gt;=G67,"Waspada","Bahaya"))</f>
+        <v>Aman</v>
       </c>
     </row>
     <row r="68" spans="3:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C68" s="58" t="s">
-        <v>417</v>
+        <v>411</v>
       </c>
       <c r="D68" s="68" t="s">
-        <v>95</v>
-      </c>
-      <c r="E68" s="64">
-        <v>0.6</v>
-      </c>
-      <c r="F68" s="72">
-        <v>0.7</v>
-      </c>
-      <c r="G68" s="72" t="s">
-        <v>416</v>
+        <v>342</v>
+      </c>
+      <c r="E68" s="62">
+        <v>0.88</v>
+      </c>
+      <c r="F68" s="71">
+        <v>0.9</v>
+      </c>
+      <c r="G68" s="71" t="s">
+        <v>412</v>
       </c>
       <c r="H68" s="70" t="str">
         <f t="shared" si="0"/>
         <v>Bahaya</v>
       </c>
     </row>
-    <row r="70" spans="3:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C70" s="116"/>
-      <c r="D70" s="116"/>
-      <c r="E70" s="116"/>
-      <c r="F70" s="116"/>
-      <c r="G70" s="116"/>
-    </row>
-    <row r="71" spans="3:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C71" s="195" t="s">
-        <v>347</v>
-      </c>
+    <row r="69" spans="3:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C69" s="58" t="s">
+        <v>413</v>
+      </c>
+      <c r="D69" s="68" t="s">
+        <v>95</v>
+      </c>
+      <c r="E69" s="64">
+        <v>0.6</v>
+      </c>
+      <c r="F69" s="72">
+        <v>0.7</v>
+      </c>
+      <c r="G69" s="72" t="s">
+        <v>412</v>
+      </c>
+      <c r="H69" s="70" t="str">
+        <f t="shared" si="0"/>
+        <v>Bahaya</v>
+      </c>
+    </row>
+    <row r="71" spans="3:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C71" s="116"/>
       <c r="D71" s="116"/>
       <c r="E71" s="116"/>
       <c r="F71" s="116"/>
       <c r="G71" s="116"/>
     </row>
     <row r="72" spans="3:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C72" s="85" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="73" spans="3:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C73" s="9" t="s">
+      <c r="C72" s="195" t="s">
+        <v>343</v>
+      </c>
+      <c r="D72" s="116"/>
+      <c r="E72" s="116"/>
+      <c r="F72" s="116"/>
+      <c r="G72" s="116"/>
+    </row>
+    <row r="73" spans="3:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C73" s="85" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="74" spans="3:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C74" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="D73" s="9" t="s">
-        <v>349</v>
-      </c>
-      <c r="E73" s="9" t="s">
+      <c r="D74" s="9" t="s">
+        <v>345</v>
+      </c>
+      <c r="E74" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="F73" s="9" t="s">
+      <c r="F74" s="9" t="s">
         <v>251</v>
       </c>
-      <c r="G73" s="9" t="s">
+      <c r="G74" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="H73" s="9" t="s">
-        <v>350</v>
-      </c>
-      <c r="I73" s="9" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="74" spans="3:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C74" s="73" t="s">
-        <v>352</v>
-      </c>
-      <c r="D74" s="74" t="s">
-        <v>353</v>
-      </c>
-      <c r="E74" s="37" t="s">
-        <v>354</v>
-      </c>
-      <c r="F74" s="66">
-        <v>4</v>
-      </c>
-      <c r="G74" s="66">
-        <v>5</v>
-      </c>
-      <c r="H74" s="10">
-        <f>INDEX(Referensi_Threshold!$D$90:$D$114,MATCH(F74*10+G74,Referensi_Threshold!$A$90:$A$114,0))</f>
-        <v>24</v>
-      </c>
-      <c r="I74" s="65" t="str">
-        <f>INDEX(Referensi_Threshold!$E$90:$E$114,MATCH(F74*10+G74,Referensi_Threshold!$A$90:$A$114,0))</f>
-        <v>High</v>
+      <c r="H74" s="9" t="s">
+        <v>346</v>
+      </c>
+      <c r="I74" s="9" t="s">
+        <v>347</v>
       </c>
     </row>
     <row r="75" spans="3:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C75" s="73" t="s">
-        <v>355</v>
+        <v>348</v>
       </c>
       <c r="D75" s="74" t="s">
-        <v>356</v>
+        <v>349</v>
       </c>
       <c r="E75" s="37" t="s">
-        <v>357</v>
+        <v>350</v>
       </c>
       <c r="F75" s="66">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G75" s="66">
         <v>5</v>
       </c>
       <c r="H75" s="10">
         <f>INDEX(Referensi_Threshold!$D$90:$D$114,MATCH(F75*10+G75,Referensi_Threshold!$A$90:$A$114,0))</f>
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I75" s="65" t="str">
         <f>INDEX(Referensi_Threshold!$E$90:$E$114,MATCH(F75*10+G75,Referensi_Threshold!$A$90:$A$114,0))</f>
@@ -7307,67 +7300,92 @@
     </row>
     <row r="76" spans="3:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C76" s="73" t="s">
-        <v>358</v>
+        <v>351</v>
       </c>
       <c r="D76" s="74" t="s">
-        <v>359</v>
+        <v>352</v>
       </c>
       <c r="E76" s="37" t="s">
-        <v>357</v>
+        <v>353</v>
       </c>
       <c r="F76" s="66">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G76" s="66">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H76" s="10">
         <f>INDEX(Referensi_Threshold!$D$90:$D$114,MATCH(F76*10+G76,Referensi_Threshold!$A$90:$A$114,0))</f>
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="I76" s="65" t="str">
         <f>INDEX(Referensi_Threshold!$E$90:$E$114,MATCH(F76*10+G76,Referensi_Threshold!$A$90:$A$114,0))</f>
-        <v>Moderate to High</v>
-      </c>
-    </row>
-    <row r="77" spans="3:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.45">
+        <v>High</v>
+      </c>
+    </row>
+    <row r="77" spans="3:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C77" s="73" t="s">
-        <v>360</v>
+        <v>354</v>
       </c>
       <c r="D77" s="74" t="s">
-        <v>361</v>
+        <v>355</v>
       </c>
       <c r="E77" s="37" t="s">
-        <v>362</v>
+        <v>353</v>
       </c>
       <c r="F77" s="66">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G77" s="66">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H77" s="10">
         <f>INDEX(Referensi_Threshold!$D$90:$D$114,MATCH(F77*10+G77,Referensi_Threshold!$A$90:$A$114,0))</f>
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="I77" s="65" t="str">
         <f>INDEX(Referensi_Threshold!$E$90:$E$114,MATCH(F77*10+G77,Referensi_Threshold!$A$90:$A$114,0))</f>
+        <v>Moderate to High</v>
+      </c>
+    </row>
+    <row r="78" spans="3:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C78" s="73" t="s">
+        <v>356</v>
+      </c>
+      <c r="D78" s="74" t="s">
+        <v>357</v>
+      </c>
+      <c r="E78" s="37" t="s">
+        <v>358</v>
+      </c>
+      <c r="F78" s="66">
+        <v>3</v>
+      </c>
+      <c r="G78" s="66">
+        <v>3</v>
+      </c>
+      <c r="H78" s="10">
+        <f>INDEX(Referensi_Threshold!$D$90:$D$114,MATCH(F78*10+G78,Referensi_Threshold!$A$90:$A$114,0))</f>
+        <v>13</v>
+      </c>
+      <c r="I78" s="65" t="str">
+        <f>INDEX(Referensi_Threshold!$E$90:$E$114,MATCH(F78*10+G78,Referensi_Threshold!$A$90:$A$114,0))</f>
         <v>Moderate</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="13">
     <mergeCell ref="C3:G3"/>
+    <mergeCell ref="C72:G72"/>
+    <mergeCell ref="C59:G59"/>
+    <mergeCell ref="C65:G65"/>
+    <mergeCell ref="C44:G44"/>
     <mergeCell ref="C71:G71"/>
+    <mergeCell ref="C7:G7"/>
+    <mergeCell ref="C35:G35"/>
+    <mergeCell ref="C51:G51"/>
     <mergeCell ref="C58:G58"/>
     <mergeCell ref="C64:G64"/>
-    <mergeCell ref="C43:G43"/>
-    <mergeCell ref="C70:G70"/>
-    <mergeCell ref="C7:G7"/>
-    <mergeCell ref="C35:G35"/>
-    <mergeCell ref="C50:G50"/>
-    <mergeCell ref="C57:G57"/>
-    <mergeCell ref="C63:G63"/>
     <mergeCell ref="C17:G17"/>
     <mergeCell ref="C26:G26"/>
   </mergeCells>
@@ -7406,8 +7424,8 @@
       <c r="G2" s="116"/>
     </row>
     <row r="3" spans="2:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B3" s="135" t="s">
-        <v>384</v>
+      <c r="B3" s="127" t="s">
+        <v>380</v>
       </c>
       <c r="C3" s="116"/>
       <c r="D3" s="116"/>
@@ -7452,7 +7470,7 @@
         <v>11</v>
       </c>
       <c r="F6" s="77" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="G6" s="77" t="s">
         <v>12</v>
@@ -7473,10 +7491,10 @@
         <v>15</v>
       </c>
       <c r="E7" s="77" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="F7" s="77" t="s">
-        <v>385</v>
+        <v>381</v>
       </c>
       <c r="G7" s="77" t="s">
         <v>16</v>
@@ -7500,7 +7518,7 @@
         <v>20</v>
       </c>
       <c r="F8" s="77" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
       <c r="G8" s="77" t="s">
         <v>21</v>
@@ -7524,7 +7542,7 @@
         <v>25</v>
       </c>
       <c r="F9" s="77" t="s">
-        <v>387</v>
+        <v>383</v>
       </c>
       <c r="G9" s="77" t="s">
         <v>26</v>
@@ -7545,10 +7563,10 @@
         <v>29</v>
       </c>
       <c r="E10" s="77" t="s">
-        <v>391</v>
+        <v>387</v>
       </c>
       <c r="F10" s="77" t="s">
-        <v>388</v>
+        <v>384</v>
       </c>
       <c r="G10" s="77" t="s">
         <v>30</v>
@@ -7566,7 +7584,7 @@
     </row>
     <row r="12" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B12" s="199" t="s">
-        <v>389</v>
+        <v>385</v>
       </c>
       <c r="C12" s="116"/>
       <c r="D12" s="116"/>
@@ -7623,7 +7641,7 @@
         <v>32</v>
       </c>
       <c r="C17" s="82">
-        <f>Input_Bulanan!F59</f>
+        <f>Input_Bulanan!F60</f>
         <v>2</v>
       </c>
       <c r="D17" s="197" t="s">
@@ -7638,7 +7656,7 @@
         <v>34</v>
       </c>
       <c r="C18" s="82">
-        <f>Input_Bulanan!F60</f>
+        <f>Input_Bulanan!F61</f>
         <v>3</v>
       </c>
       <c r="D18" s="197" t="s">
@@ -7653,7 +7671,7 @@
         <v>36</v>
       </c>
       <c r="C19" s="82">
-        <f>Input_Bulanan!F61</f>
+        <f>Input_Bulanan!F62</f>
         <v>5</v>
       </c>
       <c r="D19" s="197" t="s">
@@ -7668,7 +7686,7 @@
         <v>38</v>
       </c>
       <c r="C20" s="82">
-        <f>Input_Bulanan!F62</f>
+        <f>Input_Bulanan!F63</f>
         <v>4</v>
       </c>
       <c r="D20" s="197" t="s">
@@ -7710,105 +7728,105 @@
     </row>
     <row r="24" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B24" s="73" t="str">
-        <f>Input_Bulanan!C74</f>
+        <f>Input_Bulanan!C75</f>
         <v>C1</v>
       </c>
       <c r="C24" s="74" t="str">
-        <f>Input_Bulanan!D74</f>
+        <f>Input_Bulanan!D75</f>
         <v>Salt Supply Disruption (gangguan pasokan garam industri)</v>
       </c>
       <c r="D24" s="37" t="str">
-        <f>Input_Bulanan!E74</f>
+        <f>Input_Bulanan!E75</f>
         <v>Hulu / Supply</v>
       </c>
       <c r="E24" s="83">
-        <f>Input_Bulanan!F74</f>
+        <f>Input_Bulanan!F75</f>
         <v>4</v>
       </c>
       <c r="F24" s="83">
-        <f>Input_Bulanan!G74</f>
+        <f>Input_Bulanan!G75</f>
         <v>5</v>
       </c>
       <c r="G24" s="84" t="str">
-        <f>Input_Bulanan!H74 &amp; "  |  " &amp; Input_Bulanan!I74</f>
+        <f>Input_Bulanan!H75 &amp; "  |  " &amp; Input_Bulanan!I75</f>
         <v>24  |  High</v>
       </c>
     </row>
     <row r="25" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B25" s="73" t="str">
-        <f>Input_Bulanan!C75</f>
+        <f>Input_Bulanan!C76</f>
         <v>C2</v>
       </c>
       <c r="C25" s="74" t="str">
-        <f>Input_Bulanan!D75</f>
+        <f>Input_Bulanan!D76</f>
         <v>Commissioning Delay (keterlambatan commissioning)</v>
       </c>
       <c r="D25" s="37" t="str">
-        <f>Input_Bulanan!E75</f>
+        <f>Input_Bulanan!E76</f>
         <v>Eksekusi</v>
       </c>
       <c r="E25" s="83">
-        <f>Input_Bulanan!F75</f>
+        <f>Input_Bulanan!F76</f>
         <v>5</v>
       </c>
       <c r="F25" s="83">
-        <f>Input_Bulanan!G75</f>
+        <f>Input_Bulanan!G76</f>
         <v>5</v>
       </c>
       <c r="G25" s="84" t="str">
-        <f>Input_Bulanan!H75 &amp; "  |  " &amp; Input_Bulanan!I75</f>
+        <f>Input_Bulanan!H76 &amp; "  |  " &amp; Input_Bulanan!I76</f>
         <v>25  |  High</v>
       </c>
     </row>
     <row r="26" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B26" s="73" t="str">
-        <f>Input_Bulanan!C76</f>
+        <f>Input_Bulanan!C77</f>
         <v>C3</v>
       </c>
       <c r="C26" s="74" t="str">
-        <f>Input_Bulanan!D76</f>
+        <f>Input_Bulanan!D77</f>
         <v>EPC Interface Issue (isu EPC interface lintas kontraktor)</v>
       </c>
       <c r="D26" s="37" t="str">
-        <f>Input_Bulanan!E76</f>
+        <f>Input_Bulanan!E77</f>
         <v>Eksekusi</v>
       </c>
       <c r="E26" s="83">
-        <f>Input_Bulanan!F76</f>
+        <f>Input_Bulanan!F77</f>
         <v>4</v>
       </c>
       <c r="F26" s="83">
-        <f>Input_Bulanan!G76</f>
+        <f>Input_Bulanan!G77</f>
         <v>4</v>
       </c>
       <c r="G26" s="84" t="str">
-        <f>Input_Bulanan!H76 &amp; "  |  " &amp; Input_Bulanan!I76</f>
+        <f>Input_Bulanan!H77 &amp; "  |  " &amp; Input_Bulanan!I77</f>
         <v>19  |  Moderate to High</v>
       </c>
     </row>
     <row r="27" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B27" s="73" t="str">
-        <f>Input_Bulanan!C77</f>
+        <f>Input_Bulanan!C78</f>
         <v>C4</v>
       </c>
       <c r="C27" s="74" t="str">
-        <f>Input_Bulanan!D77</f>
+        <f>Input_Bulanan!D78</f>
         <v>Long Lead Equipment (keterlambatan peralatan utama)</v>
       </c>
       <c r="D27" s="37" t="str">
-        <f>Input_Bulanan!E77</f>
+        <f>Input_Bulanan!E78</f>
         <v>Pengadaan</v>
       </c>
       <c r="E27" s="83">
-        <f>Input_Bulanan!F77</f>
+        <f>Input_Bulanan!F78</f>
         <v>3</v>
       </c>
       <c r="F27" s="83">
-        <f>Input_Bulanan!G77</f>
+        <f>Input_Bulanan!G78</f>
         <v>3</v>
       </c>
       <c r="G27" s="84" t="str">
-        <f>Input_Bulanan!H77 &amp; "  |  " &amp; Input_Bulanan!I77</f>
+        <f>Input_Bulanan!H78 &amp; "  |  " &amp; Input_Bulanan!I78</f>
         <v>13  |  Moderate</v>
       </c>
     </row>

</xml_diff>